<commit_message>
New variables: deposit-weeks and prepay-weeks
</commit_message>
<xml_diff>
--- a/src/export/xlsx/template.xlsx
+++ b/src/export/xlsx/template.xlsx
@@ -876,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>53000</v>
+        <v>50000</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>135000</v>
+        <v>150000</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -949,30 +949,15 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Alimony per year</t>
+          <t>Income per year</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>25200</v>
+        <v>32866.8</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>£/year (counted as income)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Pension per year</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>6500</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>£/year (counted as income)</t>
+          <t>£/year (total, includes PEA)</t>
         </is>
       </c>
     </row>
@@ -998,7 +983,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>((B6+B7)/52)+B8</f>
+        <f>B6/52</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +994,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>SUM(B6:B7)+B8*52</f>
+        <f>B6</f>
         <v/>
       </c>
     </row>
@@ -1189,7 +1174,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>46296</v>
+        <v>46388</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1224,7 +1209,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Standard rate with or without nursing</t>
+          <t>Standard rate (without nursing)</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1270,37 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fees billed every N weeks, paid at the start of each period</t>
+          <t>Care home fees billed every N weeks, paid at the start of each period</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Care home deposit (weeks, returned at end)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>One-off deposit = N weeks' fee, held (illiquid) and returned in the final week</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Care home prepay weeks (paid up front)</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Weeks of fees paid up front on entry, before regular billing</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1660,12 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Means-test crossing (£60K, 03 Aug 2028)</t>
+          <t>Means-test crossing (£60K, 05 Jan 2029)</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Upper crossing (£36,750, 07 Dec 2028)</t>
+          <t>Upper crossing (£36,750, 04 May 2029)</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1782,7 @@
         <v/>
       </c>
       <c r="AC2" s="11">
-        <f>IF(MOD(A2-1,Variables!$B$30)=0,Variables!$B$30*M2,0)</f>
+        <f>IF(A2=1,MIN(Variables!$B$32,260)*M2+Variables!$B$31*Variables!$B$2,IF(MOD(A2-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A2-1))*M2,0))-IF(A2=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD2" s="12">
@@ -1892,7 +1907,7 @@
         <v/>
       </c>
       <c r="AC3" s="11">
-        <f>IF(MOD(A3-1,Variables!$B$30)=0,Variables!$B$30*M3,0)</f>
+        <f>IF(A3=1,MIN(Variables!$B$32,260)*M3+Variables!$B$31*Variables!$B$2,IF(MOD(A3-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A3-1))*M3,0))-IF(A3=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD3" s="12">
@@ -2017,7 +2032,7 @@
         <v/>
       </c>
       <c r="AC4" s="11">
-        <f>IF(MOD(A4-1,Variables!$B$30)=0,Variables!$B$30*M4,0)</f>
+        <f>IF(A4=1,MIN(Variables!$B$32,260)*M4+Variables!$B$31*Variables!$B$2,IF(MOD(A4-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A4-1))*M4,0))-IF(A4=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD4" s="12">
@@ -2142,7 +2157,7 @@
         <v/>
       </c>
       <c r="AC5" s="11">
-        <f>IF(MOD(A5-1,Variables!$B$30)=0,Variables!$B$30*M5,0)</f>
+        <f>IF(A5=1,MIN(Variables!$B$32,260)*M5+Variables!$B$31*Variables!$B$2,IF(MOD(A5-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A5-1))*M5,0))-IF(A5=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD5" s="12">
@@ -2267,7 +2282,7 @@
         <v/>
       </c>
       <c r="AC6" s="11">
-        <f>IF(MOD(A6-1,Variables!$B$30)=0,Variables!$B$30*M6,0)</f>
+        <f>IF(A6=1,MIN(Variables!$B$32,260)*M6+Variables!$B$31*Variables!$B$2,IF(MOD(A6-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A6-1))*M6,0))-IF(A6=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD6" s="12">
@@ -2392,7 +2407,7 @@
         <v/>
       </c>
       <c r="AC7" s="11">
-        <f>IF(MOD(A7-1,Variables!$B$30)=0,Variables!$B$30*M7,0)</f>
+        <f>IF(A7=1,MIN(Variables!$B$32,260)*M7+Variables!$B$31*Variables!$B$2,IF(MOD(A7-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A7-1))*M7,0))-IF(A7=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD7" s="12">
@@ -2517,7 +2532,7 @@
         <v/>
       </c>
       <c r="AC8" s="11">
-        <f>IF(MOD(A8-1,Variables!$B$30)=0,Variables!$B$30*M8,0)</f>
+        <f>IF(A8=1,MIN(Variables!$B$32,260)*M8+Variables!$B$31*Variables!$B$2,IF(MOD(A8-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A8-1))*M8,0))-IF(A8=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD8" s="12">
@@ -2642,7 +2657,7 @@
         <v/>
       </c>
       <c r="AC9" s="11">
-        <f>IF(MOD(A9-1,Variables!$B$30)=0,Variables!$B$30*M9,0)</f>
+        <f>IF(A9=1,MIN(Variables!$B$32,260)*M9+Variables!$B$31*Variables!$B$2,IF(MOD(A9-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A9-1))*M9,0))-IF(A9=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD9" s="12">
@@ -2767,7 +2782,7 @@
         <v/>
       </c>
       <c r="AC10" s="11">
-        <f>IF(MOD(A10-1,Variables!$B$30)=0,Variables!$B$30*M10,0)</f>
+        <f>IF(A10=1,MIN(Variables!$B$32,260)*M10+Variables!$B$31*Variables!$B$2,IF(MOD(A10-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A10-1))*M10,0))-IF(A10=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD10" s="12">
@@ -2892,7 +2907,7 @@
         <v/>
       </c>
       <c r="AC11" s="11">
-        <f>IF(MOD(A11-1,Variables!$B$30)=0,Variables!$B$30*M11,0)</f>
+        <f>IF(A11=1,MIN(Variables!$B$32,260)*M11+Variables!$B$31*Variables!$B$2,IF(MOD(A11-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A11-1))*M11,0))-IF(A11=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD11" s="12">
@@ -3017,7 +3032,7 @@
         <v/>
       </c>
       <c r="AC12" s="11">
-        <f>IF(MOD(A12-1,Variables!$B$30)=0,Variables!$B$30*M12,0)</f>
+        <f>IF(A12=1,MIN(Variables!$B$32,260)*M12+Variables!$B$31*Variables!$B$2,IF(MOD(A12-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A12-1))*M12,0))-IF(A12=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD12" s="12">
@@ -3142,7 +3157,7 @@
         <v/>
       </c>
       <c r="AC13" s="11">
-        <f>IF(MOD(A13-1,Variables!$B$30)=0,Variables!$B$30*M13,0)</f>
+        <f>IF(A13=1,MIN(Variables!$B$32,260)*M13+Variables!$B$31*Variables!$B$2,IF(MOD(A13-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A13-1))*M13,0))-IF(A13=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD13" s="12">
@@ -3267,7 +3282,7 @@
         <v/>
       </c>
       <c r="AC14" s="11">
-        <f>IF(MOD(A14-1,Variables!$B$30)=0,Variables!$B$30*M14,0)</f>
+        <f>IF(A14=1,MIN(Variables!$B$32,260)*M14+Variables!$B$31*Variables!$B$2,IF(MOD(A14-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A14-1))*M14,0))-IF(A14=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD14" s="12">
@@ -3392,7 +3407,7 @@
         <v/>
       </c>
       <c r="AC15" s="11">
-        <f>IF(MOD(A15-1,Variables!$B$30)=0,Variables!$B$30*M15,0)</f>
+        <f>IF(A15=1,MIN(Variables!$B$32,260)*M15+Variables!$B$31*Variables!$B$2,IF(MOD(A15-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A15-1))*M15,0))-IF(A15=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD15" s="12">
@@ -3517,7 +3532,7 @@
         <v/>
       </c>
       <c r="AC16" s="11">
-        <f>IF(MOD(A16-1,Variables!$B$30)=0,Variables!$B$30*M16,0)</f>
+        <f>IF(A16=1,MIN(Variables!$B$32,260)*M16+Variables!$B$31*Variables!$B$2,IF(MOD(A16-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A16-1))*M16,0))-IF(A16=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD16" s="12">
@@ -3642,7 +3657,7 @@
         <v/>
       </c>
       <c r="AC17" s="11">
-        <f>IF(MOD(A17-1,Variables!$B$30)=0,Variables!$B$30*M17,0)</f>
+        <f>IF(A17=1,MIN(Variables!$B$32,260)*M17+Variables!$B$31*Variables!$B$2,IF(MOD(A17-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A17-1))*M17,0))-IF(A17=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD17" s="12">
@@ -3767,7 +3782,7 @@
         <v/>
       </c>
       <c r="AC18" s="11">
-        <f>IF(MOD(A18-1,Variables!$B$30)=0,Variables!$B$30*M18,0)</f>
+        <f>IF(A18=1,MIN(Variables!$B$32,260)*M18+Variables!$B$31*Variables!$B$2,IF(MOD(A18-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A18-1))*M18,0))-IF(A18=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD18" s="12">
@@ -3892,7 +3907,7 @@
         <v/>
       </c>
       <c r="AC19" s="11">
-        <f>IF(MOD(A19-1,Variables!$B$30)=0,Variables!$B$30*M19,0)</f>
+        <f>IF(A19=1,MIN(Variables!$B$32,260)*M19+Variables!$B$31*Variables!$B$2,IF(MOD(A19-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A19-1))*M19,0))-IF(A19=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD19" s="12">
@@ -4017,7 +4032,7 @@
         <v/>
       </c>
       <c r="AC20" s="11">
-        <f>IF(MOD(A20-1,Variables!$B$30)=0,Variables!$B$30*M20,0)</f>
+        <f>IF(A20=1,MIN(Variables!$B$32,260)*M20+Variables!$B$31*Variables!$B$2,IF(MOD(A20-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A20-1))*M20,0))-IF(A20=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD20" s="12">
@@ -4142,7 +4157,7 @@
         <v/>
       </c>
       <c r="AC21" s="11">
-        <f>IF(MOD(A21-1,Variables!$B$30)=0,Variables!$B$30*M21,0)</f>
+        <f>IF(A21=1,MIN(Variables!$B$32,260)*M21+Variables!$B$31*Variables!$B$2,IF(MOD(A21-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A21-1))*M21,0))-IF(A21=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD21" s="12">
@@ -4267,7 +4282,7 @@
         <v/>
       </c>
       <c r="AC22" s="11">
-        <f>IF(MOD(A22-1,Variables!$B$30)=0,Variables!$B$30*M22,0)</f>
+        <f>IF(A22=1,MIN(Variables!$B$32,260)*M22+Variables!$B$31*Variables!$B$2,IF(MOD(A22-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A22-1))*M22,0))-IF(A22=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD22" s="12">
@@ -4392,7 +4407,7 @@
         <v/>
       </c>
       <c r="AC23" s="11">
-        <f>IF(MOD(A23-1,Variables!$B$30)=0,Variables!$B$30*M23,0)</f>
+        <f>IF(A23=1,MIN(Variables!$B$32,260)*M23+Variables!$B$31*Variables!$B$2,IF(MOD(A23-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A23-1))*M23,0))-IF(A23=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD23" s="12">
@@ -4517,7 +4532,7 @@
         <v/>
       </c>
       <c r="AC24" s="11">
-        <f>IF(MOD(A24-1,Variables!$B$30)=0,Variables!$B$30*M24,0)</f>
+        <f>IF(A24=1,MIN(Variables!$B$32,260)*M24+Variables!$B$31*Variables!$B$2,IF(MOD(A24-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A24-1))*M24,0))-IF(A24=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD24" s="12">
@@ -4642,7 +4657,7 @@
         <v/>
       </c>
       <c r="AC25" s="11">
-        <f>IF(MOD(A25-1,Variables!$B$30)=0,Variables!$B$30*M25,0)</f>
+        <f>IF(A25=1,MIN(Variables!$B$32,260)*M25+Variables!$B$31*Variables!$B$2,IF(MOD(A25-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A25-1))*M25,0))-IF(A25=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD25" s="12">
@@ -4767,7 +4782,7 @@
         <v/>
       </c>
       <c r="AC26" s="11">
-        <f>IF(MOD(A26-1,Variables!$B$30)=0,Variables!$B$30*M26,0)</f>
+        <f>IF(A26=1,MIN(Variables!$B$32,260)*M26+Variables!$B$31*Variables!$B$2,IF(MOD(A26-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A26-1))*M26,0))-IF(A26=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD26" s="12">
@@ -4892,7 +4907,7 @@
         <v/>
       </c>
       <c r="AC27" s="11">
-        <f>IF(MOD(A27-1,Variables!$B$30)=0,Variables!$B$30*M27,0)</f>
+        <f>IF(A27=1,MIN(Variables!$B$32,260)*M27+Variables!$B$31*Variables!$B$2,IF(MOD(A27-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A27-1))*M27,0))-IF(A27=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD27" s="12">
@@ -5017,7 +5032,7 @@
         <v/>
       </c>
       <c r="AC28" s="11">
-        <f>IF(MOD(A28-1,Variables!$B$30)=0,Variables!$B$30*M28,0)</f>
+        <f>IF(A28=1,MIN(Variables!$B$32,260)*M28+Variables!$B$31*Variables!$B$2,IF(MOD(A28-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A28-1))*M28,0))-IF(A28=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD28" s="12">
@@ -5142,7 +5157,7 @@
         <v/>
       </c>
       <c r="AC29" s="11">
-        <f>IF(MOD(A29-1,Variables!$B$30)=0,Variables!$B$30*M29,0)</f>
+        <f>IF(A29=1,MIN(Variables!$B$32,260)*M29+Variables!$B$31*Variables!$B$2,IF(MOD(A29-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A29-1))*M29,0))-IF(A29=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD29" s="12">
@@ -5267,7 +5282,7 @@
         <v/>
       </c>
       <c r="AC30" s="11">
-        <f>IF(MOD(A30-1,Variables!$B$30)=0,Variables!$B$30*M30,0)</f>
+        <f>IF(A30=1,MIN(Variables!$B$32,260)*M30+Variables!$B$31*Variables!$B$2,IF(MOD(A30-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A30-1))*M30,0))-IF(A30=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD30" s="12">
@@ -5392,7 +5407,7 @@
         <v/>
       </c>
       <c r="AC31" s="11">
-        <f>IF(MOD(A31-1,Variables!$B$30)=0,Variables!$B$30*M31,0)</f>
+        <f>IF(A31=1,MIN(Variables!$B$32,260)*M31+Variables!$B$31*Variables!$B$2,IF(MOD(A31-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A31-1))*M31,0))-IF(A31=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD31" s="12">
@@ -5517,7 +5532,7 @@
         <v/>
       </c>
       <c r="AC32" s="11">
-        <f>IF(MOD(A32-1,Variables!$B$30)=0,Variables!$B$30*M32,0)</f>
+        <f>IF(A32=1,MIN(Variables!$B$32,260)*M32+Variables!$B$31*Variables!$B$2,IF(MOD(A32-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A32-1))*M32,0))-IF(A32=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD32" s="12">
@@ -5642,7 +5657,7 @@
         <v/>
       </c>
       <c r="AC33" s="11">
-        <f>IF(MOD(A33-1,Variables!$B$30)=0,Variables!$B$30*M33,0)</f>
+        <f>IF(A33=1,MIN(Variables!$B$32,260)*M33+Variables!$B$31*Variables!$B$2,IF(MOD(A33-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A33-1))*M33,0))-IF(A33=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD33" s="12">
@@ -5767,7 +5782,7 @@
         <v/>
       </c>
       <c r="AC34" s="11">
-        <f>IF(MOD(A34-1,Variables!$B$30)=0,Variables!$B$30*M34,0)</f>
+        <f>IF(A34=1,MIN(Variables!$B$32,260)*M34+Variables!$B$31*Variables!$B$2,IF(MOD(A34-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A34-1))*M34,0))-IF(A34=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD34" s="12">
@@ -5892,7 +5907,7 @@
         <v/>
       </c>
       <c r="AC35" s="11">
-        <f>IF(MOD(A35-1,Variables!$B$30)=0,Variables!$B$30*M35,0)</f>
+        <f>IF(A35=1,MIN(Variables!$B$32,260)*M35+Variables!$B$31*Variables!$B$2,IF(MOD(A35-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A35-1))*M35,0))-IF(A35=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD35" s="12">
@@ -6017,7 +6032,7 @@
         <v/>
       </c>
       <c r="AC36" s="11">
-        <f>IF(MOD(A36-1,Variables!$B$30)=0,Variables!$B$30*M36,0)</f>
+        <f>IF(A36=1,MIN(Variables!$B$32,260)*M36+Variables!$B$31*Variables!$B$2,IF(MOD(A36-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A36-1))*M36,0))-IF(A36=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD36" s="12">
@@ -6142,7 +6157,7 @@
         <v/>
       </c>
       <c r="AC37" s="11">
-        <f>IF(MOD(A37-1,Variables!$B$30)=0,Variables!$B$30*M37,0)</f>
+        <f>IF(A37=1,MIN(Variables!$B$32,260)*M37+Variables!$B$31*Variables!$B$2,IF(MOD(A37-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A37-1))*M37,0))-IF(A37=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD37" s="12">
@@ -6267,7 +6282,7 @@
         <v/>
       </c>
       <c r="AC38" s="11">
-        <f>IF(MOD(A38-1,Variables!$B$30)=0,Variables!$B$30*M38,0)</f>
+        <f>IF(A38=1,MIN(Variables!$B$32,260)*M38+Variables!$B$31*Variables!$B$2,IF(MOD(A38-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A38-1))*M38,0))-IF(A38=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD38" s="12">
@@ -6392,7 +6407,7 @@
         <v/>
       </c>
       <c r="AC39" s="11">
-        <f>IF(MOD(A39-1,Variables!$B$30)=0,Variables!$B$30*M39,0)</f>
+        <f>IF(A39=1,MIN(Variables!$B$32,260)*M39+Variables!$B$31*Variables!$B$2,IF(MOD(A39-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A39-1))*M39,0))-IF(A39=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD39" s="12">
@@ -6517,7 +6532,7 @@
         <v/>
       </c>
       <c r="AC40" s="11">
-        <f>IF(MOD(A40-1,Variables!$B$30)=0,Variables!$B$30*M40,0)</f>
+        <f>IF(A40=1,MIN(Variables!$B$32,260)*M40+Variables!$B$31*Variables!$B$2,IF(MOD(A40-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A40-1))*M40,0))-IF(A40=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD40" s="12">
@@ -6642,7 +6657,7 @@
         <v/>
       </c>
       <c r="AC41" s="11">
-        <f>IF(MOD(A41-1,Variables!$B$30)=0,Variables!$B$30*M41,0)</f>
+        <f>IF(A41=1,MIN(Variables!$B$32,260)*M41+Variables!$B$31*Variables!$B$2,IF(MOD(A41-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A41-1))*M41,0))-IF(A41=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD41" s="12">
@@ -6767,7 +6782,7 @@
         <v/>
       </c>
       <c r="AC42" s="11">
-        <f>IF(MOD(A42-1,Variables!$B$30)=0,Variables!$B$30*M42,0)</f>
+        <f>IF(A42=1,MIN(Variables!$B$32,260)*M42+Variables!$B$31*Variables!$B$2,IF(MOD(A42-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A42-1))*M42,0))-IF(A42=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD42" s="12">
@@ -6892,7 +6907,7 @@
         <v/>
       </c>
       <c r="AC43" s="11">
-        <f>IF(MOD(A43-1,Variables!$B$30)=0,Variables!$B$30*M43,0)</f>
+        <f>IF(A43=1,MIN(Variables!$B$32,260)*M43+Variables!$B$31*Variables!$B$2,IF(MOD(A43-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A43-1))*M43,0))-IF(A43=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD43" s="12">
@@ -7017,7 +7032,7 @@
         <v/>
       </c>
       <c r="AC44" s="11">
-        <f>IF(MOD(A44-1,Variables!$B$30)=0,Variables!$B$30*M44,0)</f>
+        <f>IF(A44=1,MIN(Variables!$B$32,260)*M44+Variables!$B$31*Variables!$B$2,IF(MOD(A44-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A44-1))*M44,0))-IF(A44=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD44" s="12">
@@ -7142,7 +7157,7 @@
         <v/>
       </c>
       <c r="AC45" s="11">
-        <f>IF(MOD(A45-1,Variables!$B$30)=0,Variables!$B$30*M45,0)</f>
+        <f>IF(A45=1,MIN(Variables!$B$32,260)*M45+Variables!$B$31*Variables!$B$2,IF(MOD(A45-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A45-1))*M45,0))-IF(A45=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD45" s="12">
@@ -7267,7 +7282,7 @@
         <v/>
       </c>
       <c r="AC46" s="11">
-        <f>IF(MOD(A46-1,Variables!$B$30)=0,Variables!$B$30*M46,0)</f>
+        <f>IF(A46=1,MIN(Variables!$B$32,260)*M46+Variables!$B$31*Variables!$B$2,IF(MOD(A46-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A46-1))*M46,0))-IF(A46=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD46" s="12">
@@ -7392,7 +7407,7 @@
         <v/>
       </c>
       <c r="AC47" s="11">
-        <f>IF(MOD(A47-1,Variables!$B$30)=0,Variables!$B$30*M47,0)</f>
+        <f>IF(A47=1,MIN(Variables!$B$32,260)*M47+Variables!$B$31*Variables!$B$2,IF(MOD(A47-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A47-1))*M47,0))-IF(A47=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD47" s="12">
@@ -7517,7 +7532,7 @@
         <v/>
       </c>
       <c r="AC48" s="11">
-        <f>IF(MOD(A48-1,Variables!$B$30)=0,Variables!$B$30*M48,0)</f>
+        <f>IF(A48=1,MIN(Variables!$B$32,260)*M48+Variables!$B$31*Variables!$B$2,IF(MOD(A48-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A48-1))*M48,0))-IF(A48=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD48" s="12">
@@ -7642,7 +7657,7 @@
         <v/>
       </c>
       <c r="AC49" s="11">
-        <f>IF(MOD(A49-1,Variables!$B$30)=0,Variables!$B$30*M49,0)</f>
+        <f>IF(A49=1,MIN(Variables!$B$32,260)*M49+Variables!$B$31*Variables!$B$2,IF(MOD(A49-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A49-1))*M49,0))-IF(A49=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD49" s="12">
@@ -7767,7 +7782,7 @@
         <v/>
       </c>
       <c r="AC50" s="11">
-        <f>IF(MOD(A50-1,Variables!$B$30)=0,Variables!$B$30*M50,0)</f>
+        <f>IF(A50=1,MIN(Variables!$B$32,260)*M50+Variables!$B$31*Variables!$B$2,IF(MOD(A50-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A50-1))*M50,0))-IF(A50=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD50" s="12">
@@ -7892,7 +7907,7 @@
         <v/>
       </c>
       <c r="AC51" s="11">
-        <f>IF(MOD(A51-1,Variables!$B$30)=0,Variables!$B$30*M51,0)</f>
+        <f>IF(A51=1,MIN(Variables!$B$32,260)*M51+Variables!$B$31*Variables!$B$2,IF(MOD(A51-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A51-1))*M51,0))-IF(A51=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD51" s="12">
@@ -8017,7 +8032,7 @@
         <v/>
       </c>
       <c r="AC52" s="11">
-        <f>IF(MOD(A52-1,Variables!$B$30)=0,Variables!$B$30*M52,0)</f>
+        <f>IF(A52=1,MIN(Variables!$B$32,260)*M52+Variables!$B$31*Variables!$B$2,IF(MOD(A52-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A52-1))*M52,0))-IF(A52=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD52" s="12">
@@ -8142,7 +8157,7 @@
         <v/>
       </c>
       <c r="AC53" s="11">
-        <f>IF(MOD(A53-1,Variables!$B$30)=0,Variables!$B$30*M53,0)</f>
+        <f>IF(A53=1,MIN(Variables!$B$32,260)*M53+Variables!$B$31*Variables!$B$2,IF(MOD(A53-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A53-1))*M53,0))-IF(A53=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD53" s="12">
@@ -8267,7 +8282,7 @@
         <v/>
       </c>
       <c r="AC54" s="11">
-        <f>IF(MOD(A54-1,Variables!$B$30)=0,Variables!$B$30*M54,0)</f>
+        <f>IF(A54=1,MIN(Variables!$B$32,260)*M54+Variables!$B$31*Variables!$B$2,IF(MOD(A54-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A54-1))*M54,0))-IF(A54=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD54" s="12">
@@ -8392,7 +8407,7 @@
         <v/>
       </c>
       <c r="AC55" s="11">
-        <f>IF(MOD(A55-1,Variables!$B$30)=0,Variables!$B$30*M55,0)</f>
+        <f>IF(A55=1,MIN(Variables!$B$32,260)*M55+Variables!$B$31*Variables!$B$2,IF(MOD(A55-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A55-1))*M55,0))-IF(A55=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD55" s="12">
@@ -8517,7 +8532,7 @@
         <v/>
       </c>
       <c r="AC56" s="11">
-        <f>IF(MOD(A56-1,Variables!$B$30)=0,Variables!$B$30*M56,0)</f>
+        <f>IF(A56=1,MIN(Variables!$B$32,260)*M56+Variables!$B$31*Variables!$B$2,IF(MOD(A56-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A56-1))*M56,0))-IF(A56=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD56" s="12">
@@ -8642,7 +8657,7 @@
         <v/>
       </c>
       <c r="AC57" s="11">
-        <f>IF(MOD(A57-1,Variables!$B$30)=0,Variables!$B$30*M57,0)</f>
+        <f>IF(A57=1,MIN(Variables!$B$32,260)*M57+Variables!$B$31*Variables!$B$2,IF(MOD(A57-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A57-1))*M57,0))-IF(A57=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD57" s="12">
@@ -8767,7 +8782,7 @@
         <v/>
       </c>
       <c r="AC58" s="11">
-        <f>IF(MOD(A58-1,Variables!$B$30)=0,Variables!$B$30*M58,0)</f>
+        <f>IF(A58=1,MIN(Variables!$B$32,260)*M58+Variables!$B$31*Variables!$B$2,IF(MOD(A58-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A58-1))*M58,0))-IF(A58=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD58" s="12">
@@ -8892,7 +8907,7 @@
         <v/>
       </c>
       <c r="AC59" s="11">
-        <f>IF(MOD(A59-1,Variables!$B$30)=0,Variables!$B$30*M59,0)</f>
+        <f>IF(A59=1,MIN(Variables!$B$32,260)*M59+Variables!$B$31*Variables!$B$2,IF(MOD(A59-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A59-1))*M59,0))-IF(A59=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD59" s="12">
@@ -9017,7 +9032,7 @@
         <v/>
       </c>
       <c r="AC60" s="11">
-        <f>IF(MOD(A60-1,Variables!$B$30)=0,Variables!$B$30*M60,0)</f>
+        <f>IF(A60=1,MIN(Variables!$B$32,260)*M60+Variables!$B$31*Variables!$B$2,IF(MOD(A60-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A60-1))*M60,0))-IF(A60=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD60" s="12">
@@ -9142,7 +9157,7 @@
         <v/>
       </c>
       <c r="AC61" s="11">
-        <f>IF(MOD(A61-1,Variables!$B$30)=0,Variables!$B$30*M61,0)</f>
+        <f>IF(A61=1,MIN(Variables!$B$32,260)*M61+Variables!$B$31*Variables!$B$2,IF(MOD(A61-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A61-1))*M61,0))-IF(A61=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD61" s="12">
@@ -9267,7 +9282,7 @@
         <v/>
       </c>
       <c r="AC62" s="11">
-        <f>IF(MOD(A62-1,Variables!$B$30)=0,Variables!$B$30*M62,0)</f>
+        <f>IF(A62=1,MIN(Variables!$B$32,260)*M62+Variables!$B$31*Variables!$B$2,IF(MOD(A62-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A62-1))*M62,0))-IF(A62=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD62" s="12">
@@ -9392,7 +9407,7 @@
         <v/>
       </c>
       <c r="AC63" s="11">
-        <f>IF(MOD(A63-1,Variables!$B$30)=0,Variables!$B$30*M63,0)</f>
+        <f>IF(A63=1,MIN(Variables!$B$32,260)*M63+Variables!$B$31*Variables!$B$2,IF(MOD(A63-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A63-1))*M63,0))-IF(A63=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD63" s="12">
@@ -9517,7 +9532,7 @@
         <v/>
       </c>
       <c r="AC64" s="11">
-        <f>IF(MOD(A64-1,Variables!$B$30)=0,Variables!$B$30*M64,0)</f>
+        <f>IF(A64=1,MIN(Variables!$B$32,260)*M64+Variables!$B$31*Variables!$B$2,IF(MOD(A64-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A64-1))*M64,0))-IF(A64=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD64" s="12">
@@ -9642,7 +9657,7 @@
         <v/>
       </c>
       <c r="AC65" s="11">
-        <f>IF(MOD(A65-1,Variables!$B$30)=0,Variables!$B$30*M65,0)</f>
+        <f>IF(A65=1,MIN(Variables!$B$32,260)*M65+Variables!$B$31*Variables!$B$2,IF(MOD(A65-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A65-1))*M65,0))-IF(A65=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD65" s="12">
@@ -9767,7 +9782,7 @@
         <v/>
       </c>
       <c r="AC66" s="11">
-        <f>IF(MOD(A66-1,Variables!$B$30)=0,Variables!$B$30*M66,0)</f>
+        <f>IF(A66=1,MIN(Variables!$B$32,260)*M66+Variables!$B$31*Variables!$B$2,IF(MOD(A66-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A66-1))*M66,0))-IF(A66=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD66" s="12">
@@ -9892,7 +9907,7 @@
         <v/>
       </c>
       <c r="AC67" s="11">
-        <f>IF(MOD(A67-1,Variables!$B$30)=0,Variables!$B$30*M67,0)</f>
+        <f>IF(A67=1,MIN(Variables!$B$32,260)*M67+Variables!$B$31*Variables!$B$2,IF(MOD(A67-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A67-1))*M67,0))-IF(A67=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD67" s="12">
@@ -10017,7 +10032,7 @@
         <v/>
       </c>
       <c r="AC68" s="11">
-        <f>IF(MOD(A68-1,Variables!$B$30)=0,Variables!$B$30*M68,0)</f>
+        <f>IF(A68=1,MIN(Variables!$B$32,260)*M68+Variables!$B$31*Variables!$B$2,IF(MOD(A68-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A68-1))*M68,0))-IF(A68=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD68" s="12">
@@ -10142,7 +10157,7 @@
         <v/>
       </c>
       <c r="AC69" s="11">
-        <f>IF(MOD(A69-1,Variables!$B$30)=0,Variables!$B$30*M69,0)</f>
+        <f>IF(A69=1,MIN(Variables!$B$32,260)*M69+Variables!$B$31*Variables!$B$2,IF(MOD(A69-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A69-1))*M69,0))-IF(A69=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD69" s="12">
@@ -10267,7 +10282,7 @@
         <v/>
       </c>
       <c r="AC70" s="11">
-        <f>IF(MOD(A70-1,Variables!$B$30)=0,Variables!$B$30*M70,0)</f>
+        <f>IF(A70=1,MIN(Variables!$B$32,260)*M70+Variables!$B$31*Variables!$B$2,IF(MOD(A70-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A70-1))*M70,0))-IF(A70=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD70" s="12">
@@ -10392,7 +10407,7 @@
         <v/>
       </c>
       <c r="AC71" s="11">
-        <f>IF(MOD(A71-1,Variables!$B$30)=0,Variables!$B$30*M71,0)</f>
+        <f>IF(A71=1,MIN(Variables!$B$32,260)*M71+Variables!$B$31*Variables!$B$2,IF(MOD(A71-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A71-1))*M71,0))-IF(A71=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD71" s="12">
@@ -10517,7 +10532,7 @@
         <v/>
       </c>
       <c r="AC72" s="11">
-        <f>IF(MOD(A72-1,Variables!$B$30)=0,Variables!$B$30*M72,0)</f>
+        <f>IF(A72=1,MIN(Variables!$B$32,260)*M72+Variables!$B$31*Variables!$B$2,IF(MOD(A72-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A72-1))*M72,0))-IF(A72=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD72" s="12">
@@ -10642,7 +10657,7 @@
         <v/>
       </c>
       <c r="AC73" s="11">
-        <f>IF(MOD(A73-1,Variables!$B$30)=0,Variables!$B$30*M73,0)</f>
+        <f>IF(A73=1,MIN(Variables!$B$32,260)*M73+Variables!$B$31*Variables!$B$2,IF(MOD(A73-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A73-1))*M73,0))-IF(A73=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD73" s="12">
@@ -10767,7 +10782,7 @@
         <v/>
       </c>
       <c r="AC74" s="11">
-        <f>IF(MOD(A74-1,Variables!$B$30)=0,Variables!$B$30*M74,0)</f>
+        <f>IF(A74=1,MIN(Variables!$B$32,260)*M74+Variables!$B$31*Variables!$B$2,IF(MOD(A74-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A74-1))*M74,0))-IF(A74=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD74" s="12">
@@ -10892,7 +10907,7 @@
         <v/>
       </c>
       <c r="AC75" s="11">
-        <f>IF(MOD(A75-1,Variables!$B$30)=0,Variables!$B$30*M75,0)</f>
+        <f>IF(A75=1,MIN(Variables!$B$32,260)*M75+Variables!$B$31*Variables!$B$2,IF(MOD(A75-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A75-1))*M75,0))-IF(A75=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD75" s="12">
@@ -11017,7 +11032,7 @@
         <v/>
       </c>
       <c r="AC76" s="11">
-        <f>IF(MOD(A76-1,Variables!$B$30)=0,Variables!$B$30*M76,0)</f>
+        <f>IF(A76=1,MIN(Variables!$B$32,260)*M76+Variables!$B$31*Variables!$B$2,IF(MOD(A76-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A76-1))*M76,0))-IF(A76=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD76" s="12">
@@ -11142,7 +11157,7 @@
         <v/>
       </c>
       <c r="AC77" s="11">
-        <f>IF(MOD(A77-1,Variables!$B$30)=0,Variables!$B$30*M77,0)</f>
+        <f>IF(A77=1,MIN(Variables!$B$32,260)*M77+Variables!$B$31*Variables!$B$2,IF(MOD(A77-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A77-1))*M77,0))-IF(A77=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD77" s="12">
@@ -11267,7 +11282,7 @@
         <v/>
       </c>
       <c r="AC78" s="11">
-        <f>IF(MOD(A78-1,Variables!$B$30)=0,Variables!$B$30*M78,0)</f>
+        <f>IF(A78=1,MIN(Variables!$B$32,260)*M78+Variables!$B$31*Variables!$B$2,IF(MOD(A78-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A78-1))*M78,0))-IF(A78=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD78" s="12">
@@ -11392,7 +11407,7 @@
         <v/>
       </c>
       <c r="AC79" s="11">
-        <f>IF(MOD(A79-1,Variables!$B$30)=0,Variables!$B$30*M79,0)</f>
+        <f>IF(A79=1,MIN(Variables!$B$32,260)*M79+Variables!$B$31*Variables!$B$2,IF(MOD(A79-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A79-1))*M79,0))-IF(A79=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD79" s="12">
@@ -11517,7 +11532,7 @@
         <v/>
       </c>
       <c r="AC80" s="11">
-        <f>IF(MOD(A80-1,Variables!$B$30)=0,Variables!$B$30*M80,0)</f>
+        <f>IF(A80=1,MIN(Variables!$B$32,260)*M80+Variables!$B$31*Variables!$B$2,IF(MOD(A80-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A80-1))*M80,0))-IF(A80=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD80" s="12">
@@ -11642,7 +11657,7 @@
         <v/>
       </c>
       <c r="AC81" s="11">
-        <f>IF(MOD(A81-1,Variables!$B$30)=0,Variables!$B$30*M81,0)</f>
+        <f>IF(A81=1,MIN(Variables!$B$32,260)*M81+Variables!$B$31*Variables!$B$2,IF(MOD(A81-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A81-1))*M81,0))-IF(A81=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD81" s="12">
@@ -11767,7 +11782,7 @@
         <v/>
       </c>
       <c r="AC82" s="11">
-        <f>IF(MOD(A82-1,Variables!$B$30)=0,Variables!$B$30*M82,0)</f>
+        <f>IF(A82=1,MIN(Variables!$B$32,260)*M82+Variables!$B$31*Variables!$B$2,IF(MOD(A82-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A82-1))*M82,0))-IF(A82=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD82" s="12">
@@ -11892,7 +11907,7 @@
         <v/>
       </c>
       <c r="AC83" s="11">
-        <f>IF(MOD(A83-1,Variables!$B$30)=0,Variables!$B$30*M83,0)</f>
+        <f>IF(A83=1,MIN(Variables!$B$32,260)*M83+Variables!$B$31*Variables!$B$2,IF(MOD(A83-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A83-1))*M83,0))-IF(A83=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD83" s="12">
@@ -12017,7 +12032,7 @@
         <v/>
       </c>
       <c r="AC84" s="11">
-        <f>IF(MOD(A84-1,Variables!$B$30)=0,Variables!$B$30*M84,0)</f>
+        <f>IF(A84=1,MIN(Variables!$B$32,260)*M84+Variables!$B$31*Variables!$B$2,IF(MOD(A84-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A84-1))*M84,0))-IF(A84=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD84" s="12">
@@ -12142,7 +12157,7 @@
         <v/>
       </c>
       <c r="AC85" s="11">
-        <f>IF(MOD(A85-1,Variables!$B$30)=0,Variables!$B$30*M85,0)</f>
+        <f>IF(A85=1,MIN(Variables!$B$32,260)*M85+Variables!$B$31*Variables!$B$2,IF(MOD(A85-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A85-1))*M85,0))-IF(A85=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD85" s="12">
@@ -12267,7 +12282,7 @@
         <v/>
       </c>
       <c r="AC86" s="11">
-        <f>IF(MOD(A86-1,Variables!$B$30)=0,Variables!$B$30*M86,0)</f>
+        <f>IF(A86=1,MIN(Variables!$B$32,260)*M86+Variables!$B$31*Variables!$B$2,IF(MOD(A86-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A86-1))*M86,0))-IF(A86=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD86" s="12">
@@ -12392,7 +12407,7 @@
         <v/>
       </c>
       <c r="AC87" s="11">
-        <f>IF(MOD(A87-1,Variables!$B$30)=0,Variables!$B$30*M87,0)</f>
+        <f>IF(A87=1,MIN(Variables!$B$32,260)*M87+Variables!$B$31*Variables!$B$2,IF(MOD(A87-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A87-1))*M87,0))-IF(A87=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD87" s="12">
@@ -12517,7 +12532,7 @@
         <v/>
       </c>
       <c r="AC88" s="11">
-        <f>IF(MOD(A88-1,Variables!$B$30)=0,Variables!$B$30*M88,0)</f>
+        <f>IF(A88=1,MIN(Variables!$B$32,260)*M88+Variables!$B$31*Variables!$B$2,IF(MOD(A88-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A88-1))*M88,0))-IF(A88=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD88" s="12">
@@ -12642,7 +12657,7 @@
         <v/>
       </c>
       <c r="AC89" s="11">
-        <f>IF(MOD(A89-1,Variables!$B$30)=0,Variables!$B$30*M89,0)</f>
+        <f>IF(A89=1,MIN(Variables!$B$32,260)*M89+Variables!$B$31*Variables!$B$2,IF(MOD(A89-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A89-1))*M89,0))-IF(A89=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD89" s="12">
@@ -12767,7 +12782,7 @@
         <v/>
       </c>
       <c r="AC90" s="11">
-        <f>IF(MOD(A90-1,Variables!$B$30)=0,Variables!$B$30*M90,0)</f>
+        <f>IF(A90=1,MIN(Variables!$B$32,260)*M90+Variables!$B$31*Variables!$B$2,IF(MOD(A90-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A90-1))*M90,0))-IF(A90=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD90" s="12">
@@ -12892,7 +12907,7 @@
         <v/>
       </c>
       <c r="AC91" s="11">
-        <f>IF(MOD(A91-1,Variables!$B$30)=0,Variables!$B$30*M91,0)</f>
+        <f>IF(A91=1,MIN(Variables!$B$32,260)*M91+Variables!$B$31*Variables!$B$2,IF(MOD(A91-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A91-1))*M91,0))-IF(A91=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD91" s="12">
@@ -13017,7 +13032,7 @@
         <v/>
       </c>
       <c r="AC92" s="11">
-        <f>IF(MOD(A92-1,Variables!$B$30)=0,Variables!$B$30*M92,0)</f>
+        <f>IF(A92=1,MIN(Variables!$B$32,260)*M92+Variables!$B$31*Variables!$B$2,IF(MOD(A92-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A92-1))*M92,0))-IF(A92=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD92" s="12">
@@ -13142,7 +13157,7 @@
         <v/>
       </c>
       <c r="AC93" s="11">
-        <f>IF(MOD(A93-1,Variables!$B$30)=0,Variables!$B$30*M93,0)</f>
+        <f>IF(A93=1,MIN(Variables!$B$32,260)*M93+Variables!$B$31*Variables!$B$2,IF(MOD(A93-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A93-1))*M93,0))-IF(A93=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD93" s="12">
@@ -13267,7 +13282,7 @@
         <v/>
       </c>
       <c r="AC94" s="11">
-        <f>IF(MOD(A94-1,Variables!$B$30)=0,Variables!$B$30*M94,0)</f>
+        <f>IF(A94=1,MIN(Variables!$B$32,260)*M94+Variables!$B$31*Variables!$B$2,IF(MOD(A94-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A94-1))*M94,0))-IF(A94=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD94" s="12">
@@ -13392,7 +13407,7 @@
         <v/>
       </c>
       <c r="AC95" s="11">
-        <f>IF(MOD(A95-1,Variables!$B$30)=0,Variables!$B$30*M95,0)</f>
+        <f>IF(A95=1,MIN(Variables!$B$32,260)*M95+Variables!$B$31*Variables!$B$2,IF(MOD(A95-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A95-1))*M95,0))-IF(A95=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD95" s="12">
@@ -13517,7 +13532,7 @@
         <v/>
       </c>
       <c r="AC96" s="11">
-        <f>IF(MOD(A96-1,Variables!$B$30)=0,Variables!$B$30*M96,0)</f>
+        <f>IF(A96=1,MIN(Variables!$B$32,260)*M96+Variables!$B$31*Variables!$B$2,IF(MOD(A96-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A96-1))*M96,0))-IF(A96=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD96" s="12">
@@ -13642,7 +13657,7 @@
         <v/>
       </c>
       <c r="AC97" s="11">
-        <f>IF(MOD(A97-1,Variables!$B$30)=0,Variables!$B$30*M97,0)</f>
+        <f>IF(A97=1,MIN(Variables!$B$32,260)*M97+Variables!$B$31*Variables!$B$2,IF(MOD(A97-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A97-1))*M97,0))-IF(A97=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD97" s="12">
@@ -13767,7 +13782,7 @@
         <v/>
       </c>
       <c r="AC98" s="11">
-        <f>IF(MOD(A98-1,Variables!$B$30)=0,Variables!$B$30*M98,0)</f>
+        <f>IF(A98=1,MIN(Variables!$B$32,260)*M98+Variables!$B$31*Variables!$B$2,IF(MOD(A98-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A98-1))*M98,0))-IF(A98=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD98" s="12">
@@ -13892,7 +13907,7 @@
         <v/>
       </c>
       <c r="AC99" s="11">
-        <f>IF(MOD(A99-1,Variables!$B$30)=0,Variables!$B$30*M99,0)</f>
+        <f>IF(A99=1,MIN(Variables!$B$32,260)*M99+Variables!$B$31*Variables!$B$2,IF(MOD(A99-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A99-1))*M99,0))-IF(A99=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD99" s="12">
@@ -14017,7 +14032,7 @@
         <v/>
       </c>
       <c r="AC100" s="11">
-        <f>IF(MOD(A100-1,Variables!$B$30)=0,Variables!$B$30*M100,0)</f>
+        <f>IF(A100=1,MIN(Variables!$B$32,260)*M100+Variables!$B$31*Variables!$B$2,IF(MOD(A100-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A100-1))*M100,0))-IF(A100=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD100" s="12">
@@ -14142,7 +14157,7 @@
         <v/>
       </c>
       <c r="AC101" s="11">
-        <f>IF(MOD(A101-1,Variables!$B$30)=0,Variables!$B$30*M101,0)</f>
+        <f>IF(A101=1,MIN(Variables!$B$32,260)*M101+Variables!$B$31*Variables!$B$2,IF(MOD(A101-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A101-1))*M101,0))-IF(A101=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD101" s="12">
@@ -14267,7 +14282,7 @@
         <v/>
       </c>
       <c r="AC102" s="11">
-        <f>IF(MOD(A102-1,Variables!$B$30)=0,Variables!$B$30*M102,0)</f>
+        <f>IF(A102=1,MIN(Variables!$B$32,260)*M102+Variables!$B$31*Variables!$B$2,IF(MOD(A102-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A102-1))*M102,0))-IF(A102=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD102" s="12">
@@ -14392,7 +14407,7 @@
         <v/>
       </c>
       <c r="AC103" s="11">
-        <f>IF(MOD(A103-1,Variables!$B$30)=0,Variables!$B$30*M103,0)</f>
+        <f>IF(A103=1,MIN(Variables!$B$32,260)*M103+Variables!$B$31*Variables!$B$2,IF(MOD(A103-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A103-1))*M103,0))-IF(A103=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD103" s="12">
@@ -14517,7 +14532,7 @@
         <v/>
       </c>
       <c r="AC104" s="11">
-        <f>IF(MOD(A104-1,Variables!$B$30)=0,Variables!$B$30*M104,0)</f>
+        <f>IF(A104=1,MIN(Variables!$B$32,260)*M104+Variables!$B$31*Variables!$B$2,IF(MOD(A104-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A104-1))*M104,0))-IF(A104=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD104" s="12">
@@ -14642,7 +14657,7 @@
         <v/>
       </c>
       <c r="AC105" s="11">
-        <f>IF(MOD(A105-1,Variables!$B$30)=0,Variables!$B$30*M105,0)</f>
+        <f>IF(A105=1,MIN(Variables!$B$32,260)*M105+Variables!$B$31*Variables!$B$2,IF(MOD(A105-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A105-1))*M105,0))-IF(A105=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD105" s="12">
@@ -14767,7 +14782,7 @@
         <v/>
       </c>
       <c r="AC106" s="11">
-        <f>IF(MOD(A106-1,Variables!$B$30)=0,Variables!$B$30*M106,0)</f>
+        <f>IF(A106=1,MIN(Variables!$B$32,260)*M106+Variables!$B$31*Variables!$B$2,IF(MOD(A106-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A106-1))*M106,0))-IF(A106=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD106" s="12">
@@ -14892,7 +14907,7 @@
         <v/>
       </c>
       <c r="AC107" s="11">
-        <f>IF(MOD(A107-1,Variables!$B$30)=0,Variables!$B$30*M107,0)</f>
+        <f>IF(A107=1,MIN(Variables!$B$32,260)*M107+Variables!$B$31*Variables!$B$2,IF(MOD(A107-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A107-1))*M107,0))-IF(A107=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD107" s="12">
@@ -15017,7 +15032,7 @@
         <v/>
       </c>
       <c r="AC108" s="11">
-        <f>IF(MOD(A108-1,Variables!$B$30)=0,Variables!$B$30*M108,0)</f>
+        <f>IF(A108=1,MIN(Variables!$B$32,260)*M108+Variables!$B$31*Variables!$B$2,IF(MOD(A108-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A108-1))*M108,0))-IF(A108=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD108" s="12">
@@ -15142,7 +15157,7 @@
         <v/>
       </c>
       <c r="AC109" s="11">
-        <f>IF(MOD(A109-1,Variables!$B$30)=0,Variables!$B$30*M109,0)</f>
+        <f>IF(A109=1,MIN(Variables!$B$32,260)*M109+Variables!$B$31*Variables!$B$2,IF(MOD(A109-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A109-1))*M109,0))-IF(A109=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD109" s="12">
@@ -15267,7 +15282,7 @@
         <v/>
       </c>
       <c r="AC110" s="11">
-        <f>IF(MOD(A110-1,Variables!$B$30)=0,Variables!$B$30*M110,0)</f>
+        <f>IF(A110=1,MIN(Variables!$B$32,260)*M110+Variables!$B$31*Variables!$B$2,IF(MOD(A110-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A110-1))*M110,0))-IF(A110=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD110" s="12">
@@ -15392,7 +15407,7 @@
         <v/>
       </c>
       <c r="AC111" s="11">
-        <f>IF(MOD(A111-1,Variables!$B$30)=0,Variables!$B$30*M111,0)</f>
+        <f>IF(A111=1,MIN(Variables!$B$32,260)*M111+Variables!$B$31*Variables!$B$2,IF(MOD(A111-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A111-1))*M111,0))-IF(A111=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD111" s="12">
@@ -15517,7 +15532,7 @@
         <v/>
       </c>
       <c r="AC112" s="11">
-        <f>IF(MOD(A112-1,Variables!$B$30)=0,Variables!$B$30*M112,0)</f>
+        <f>IF(A112=1,MIN(Variables!$B$32,260)*M112+Variables!$B$31*Variables!$B$2,IF(MOD(A112-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A112-1))*M112,0))-IF(A112=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD112" s="12">
@@ -15642,7 +15657,7 @@
         <v/>
       </c>
       <c r="AC113" s="11">
-        <f>IF(MOD(A113-1,Variables!$B$30)=0,Variables!$B$30*M113,0)</f>
+        <f>IF(A113=1,MIN(Variables!$B$32,260)*M113+Variables!$B$31*Variables!$B$2,IF(MOD(A113-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A113-1))*M113,0))-IF(A113=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD113" s="12">
@@ -15767,7 +15782,7 @@
         <v/>
       </c>
       <c r="AC114" s="11">
-        <f>IF(MOD(A114-1,Variables!$B$30)=0,Variables!$B$30*M114,0)</f>
+        <f>IF(A114=1,MIN(Variables!$B$32,260)*M114+Variables!$B$31*Variables!$B$2,IF(MOD(A114-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A114-1))*M114,0))-IF(A114=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD114" s="12">
@@ -15892,7 +15907,7 @@
         <v/>
       </c>
       <c r="AC115" s="11">
-        <f>IF(MOD(A115-1,Variables!$B$30)=0,Variables!$B$30*M115,0)</f>
+        <f>IF(A115=1,MIN(Variables!$B$32,260)*M115+Variables!$B$31*Variables!$B$2,IF(MOD(A115-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A115-1))*M115,0))-IF(A115=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD115" s="12">
@@ -16017,7 +16032,7 @@
         <v/>
       </c>
       <c r="AC116" s="11">
-        <f>IF(MOD(A116-1,Variables!$B$30)=0,Variables!$B$30*M116,0)</f>
+        <f>IF(A116=1,MIN(Variables!$B$32,260)*M116+Variables!$B$31*Variables!$B$2,IF(MOD(A116-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A116-1))*M116,0))-IF(A116=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD116" s="12">
@@ -16142,7 +16157,7 @@
         <v/>
       </c>
       <c r="AC117" s="11">
-        <f>IF(MOD(A117-1,Variables!$B$30)=0,Variables!$B$30*M117,0)</f>
+        <f>IF(A117=1,MIN(Variables!$B$32,260)*M117+Variables!$B$31*Variables!$B$2,IF(MOD(A117-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A117-1))*M117,0))-IF(A117=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD117" s="12">
@@ -16267,7 +16282,7 @@
         <v/>
       </c>
       <c r="AC118" s="11">
-        <f>IF(MOD(A118-1,Variables!$B$30)=0,Variables!$B$30*M118,0)</f>
+        <f>IF(A118=1,MIN(Variables!$B$32,260)*M118+Variables!$B$31*Variables!$B$2,IF(MOD(A118-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A118-1))*M118,0))-IF(A118=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD118" s="12">
@@ -16392,7 +16407,7 @@
         <v/>
       </c>
       <c r="AC119" s="11">
-        <f>IF(MOD(A119-1,Variables!$B$30)=0,Variables!$B$30*M119,0)</f>
+        <f>IF(A119=1,MIN(Variables!$B$32,260)*M119+Variables!$B$31*Variables!$B$2,IF(MOD(A119-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A119-1))*M119,0))-IF(A119=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD119" s="12">
@@ -16517,7 +16532,7 @@
         <v/>
       </c>
       <c r="AC120" s="11">
-        <f>IF(MOD(A120-1,Variables!$B$30)=0,Variables!$B$30*M120,0)</f>
+        <f>IF(A120=1,MIN(Variables!$B$32,260)*M120+Variables!$B$31*Variables!$B$2,IF(MOD(A120-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A120-1))*M120,0))-IF(A120=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD120" s="12">
@@ -16642,7 +16657,7 @@
         <v/>
       </c>
       <c r="AC121" s="11">
-        <f>IF(MOD(A121-1,Variables!$B$30)=0,Variables!$B$30*M121,0)</f>
+        <f>IF(A121=1,MIN(Variables!$B$32,260)*M121+Variables!$B$31*Variables!$B$2,IF(MOD(A121-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A121-1))*M121,0))-IF(A121=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD121" s="12">
@@ -16767,7 +16782,7 @@
         <v/>
       </c>
       <c r="AC122" s="11">
-        <f>IF(MOD(A122-1,Variables!$B$30)=0,Variables!$B$30*M122,0)</f>
+        <f>IF(A122=1,MIN(Variables!$B$32,260)*M122+Variables!$B$31*Variables!$B$2,IF(MOD(A122-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A122-1))*M122,0))-IF(A122=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD122" s="12">
@@ -16892,7 +16907,7 @@
         <v/>
       </c>
       <c r="AC123" s="11">
-        <f>IF(MOD(A123-1,Variables!$B$30)=0,Variables!$B$30*M123,0)</f>
+        <f>IF(A123=1,MIN(Variables!$B$32,260)*M123+Variables!$B$31*Variables!$B$2,IF(MOD(A123-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A123-1))*M123,0))-IF(A123=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD123" s="12">
@@ -17017,7 +17032,7 @@
         <v/>
       </c>
       <c r="AC124" s="11">
-        <f>IF(MOD(A124-1,Variables!$B$30)=0,Variables!$B$30*M124,0)</f>
+        <f>IF(A124=1,MIN(Variables!$B$32,260)*M124+Variables!$B$31*Variables!$B$2,IF(MOD(A124-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A124-1))*M124,0))-IF(A124=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD124" s="12">
@@ -17142,7 +17157,7 @@
         <v/>
       </c>
       <c r="AC125" s="11">
-        <f>IF(MOD(A125-1,Variables!$B$30)=0,Variables!$B$30*M125,0)</f>
+        <f>IF(A125=1,MIN(Variables!$B$32,260)*M125+Variables!$B$31*Variables!$B$2,IF(MOD(A125-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A125-1))*M125,0))-IF(A125=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD125" s="12">
@@ -17267,7 +17282,7 @@
         <v/>
       </c>
       <c r="AC126" s="11">
-        <f>IF(MOD(A126-1,Variables!$B$30)=0,Variables!$B$30*M126,0)</f>
+        <f>IF(A126=1,MIN(Variables!$B$32,260)*M126+Variables!$B$31*Variables!$B$2,IF(MOD(A126-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A126-1))*M126,0))-IF(A126=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD126" s="12">
@@ -17392,7 +17407,7 @@
         <v/>
       </c>
       <c r="AC127" s="11">
-        <f>IF(MOD(A127-1,Variables!$B$30)=0,Variables!$B$30*M127,0)</f>
+        <f>IF(A127=1,MIN(Variables!$B$32,260)*M127+Variables!$B$31*Variables!$B$2,IF(MOD(A127-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A127-1))*M127,0))-IF(A127=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD127" s="12">
@@ -17517,7 +17532,7 @@
         <v/>
       </c>
       <c r="AC128" s="11">
-        <f>IF(MOD(A128-1,Variables!$B$30)=0,Variables!$B$30*M128,0)</f>
+        <f>IF(A128=1,MIN(Variables!$B$32,260)*M128+Variables!$B$31*Variables!$B$2,IF(MOD(A128-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A128-1))*M128,0))-IF(A128=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD128" s="12">
@@ -17642,7 +17657,7 @@
         <v/>
       </c>
       <c r="AC129" s="11">
-        <f>IF(MOD(A129-1,Variables!$B$30)=0,Variables!$B$30*M129,0)</f>
+        <f>IF(A129=1,MIN(Variables!$B$32,260)*M129+Variables!$B$31*Variables!$B$2,IF(MOD(A129-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A129-1))*M129,0))-IF(A129=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD129" s="12">
@@ -17767,7 +17782,7 @@
         <v/>
       </c>
       <c r="AC130" s="11">
-        <f>IF(MOD(A130-1,Variables!$B$30)=0,Variables!$B$30*M130,0)</f>
+        <f>IF(A130=1,MIN(Variables!$B$32,260)*M130+Variables!$B$31*Variables!$B$2,IF(MOD(A130-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A130-1))*M130,0))-IF(A130=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD130" s="12">
@@ -17892,7 +17907,7 @@
         <v/>
       </c>
       <c r="AC131" s="11">
-        <f>IF(MOD(A131-1,Variables!$B$30)=0,Variables!$B$30*M131,0)</f>
+        <f>IF(A131=1,MIN(Variables!$B$32,260)*M131+Variables!$B$31*Variables!$B$2,IF(MOD(A131-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A131-1))*M131,0))-IF(A131=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD131" s="12">
@@ -18017,7 +18032,7 @@
         <v/>
       </c>
       <c r="AC132" s="11">
-        <f>IF(MOD(A132-1,Variables!$B$30)=0,Variables!$B$30*M132,0)</f>
+        <f>IF(A132=1,MIN(Variables!$B$32,260)*M132+Variables!$B$31*Variables!$B$2,IF(MOD(A132-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A132-1))*M132,0))-IF(A132=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD132" s="12">
@@ -18142,7 +18157,7 @@
         <v/>
       </c>
       <c r="AC133" s="11">
-        <f>IF(MOD(A133-1,Variables!$B$30)=0,Variables!$B$30*M133,0)</f>
+        <f>IF(A133=1,MIN(Variables!$B$32,260)*M133+Variables!$B$31*Variables!$B$2,IF(MOD(A133-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A133-1))*M133,0))-IF(A133=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD133" s="12">
@@ -18267,7 +18282,7 @@
         <v/>
       </c>
       <c r="AC134" s="11">
-        <f>IF(MOD(A134-1,Variables!$B$30)=0,Variables!$B$30*M134,0)</f>
+        <f>IF(A134=1,MIN(Variables!$B$32,260)*M134+Variables!$B$31*Variables!$B$2,IF(MOD(A134-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A134-1))*M134,0))-IF(A134=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD134" s="12">
@@ -18392,7 +18407,7 @@
         <v/>
       </c>
       <c r="AC135" s="11">
-        <f>IF(MOD(A135-1,Variables!$B$30)=0,Variables!$B$30*M135,0)</f>
+        <f>IF(A135=1,MIN(Variables!$B$32,260)*M135+Variables!$B$31*Variables!$B$2,IF(MOD(A135-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A135-1))*M135,0))-IF(A135=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD135" s="12">
@@ -18517,7 +18532,7 @@
         <v/>
       </c>
       <c r="AC136" s="11">
-        <f>IF(MOD(A136-1,Variables!$B$30)=0,Variables!$B$30*M136,0)</f>
+        <f>IF(A136=1,MIN(Variables!$B$32,260)*M136+Variables!$B$31*Variables!$B$2,IF(MOD(A136-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A136-1))*M136,0))-IF(A136=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD136" s="12">
@@ -18642,7 +18657,7 @@
         <v/>
       </c>
       <c r="AC137" s="11">
-        <f>IF(MOD(A137-1,Variables!$B$30)=0,Variables!$B$30*M137,0)</f>
+        <f>IF(A137=1,MIN(Variables!$B$32,260)*M137+Variables!$B$31*Variables!$B$2,IF(MOD(A137-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A137-1))*M137,0))-IF(A137=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD137" s="12">
@@ -18767,7 +18782,7 @@
         <v/>
       </c>
       <c r="AC138" s="11">
-        <f>IF(MOD(A138-1,Variables!$B$30)=0,Variables!$B$30*M138,0)</f>
+        <f>IF(A138=1,MIN(Variables!$B$32,260)*M138+Variables!$B$31*Variables!$B$2,IF(MOD(A138-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A138-1))*M138,0))-IF(A138=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD138" s="12">
@@ -18892,7 +18907,7 @@
         <v/>
       </c>
       <c r="AC139" s="11">
-        <f>IF(MOD(A139-1,Variables!$B$30)=0,Variables!$B$30*M139,0)</f>
+        <f>IF(A139=1,MIN(Variables!$B$32,260)*M139+Variables!$B$31*Variables!$B$2,IF(MOD(A139-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A139-1))*M139,0))-IF(A139=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD139" s="12">
@@ -19017,7 +19032,7 @@
         <v/>
       </c>
       <c r="AC140" s="11">
-        <f>IF(MOD(A140-1,Variables!$B$30)=0,Variables!$B$30*M140,0)</f>
+        <f>IF(A140=1,MIN(Variables!$B$32,260)*M140+Variables!$B$31*Variables!$B$2,IF(MOD(A140-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A140-1))*M140,0))-IF(A140=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD140" s="12">
@@ -19142,7 +19157,7 @@
         <v/>
       </c>
       <c r="AC141" s="11">
-        <f>IF(MOD(A141-1,Variables!$B$30)=0,Variables!$B$30*M141,0)</f>
+        <f>IF(A141=1,MIN(Variables!$B$32,260)*M141+Variables!$B$31*Variables!$B$2,IF(MOD(A141-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A141-1))*M141,0))-IF(A141=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD141" s="12">
@@ -19267,7 +19282,7 @@
         <v/>
       </c>
       <c r="AC142" s="11">
-        <f>IF(MOD(A142-1,Variables!$B$30)=0,Variables!$B$30*M142,0)</f>
+        <f>IF(A142=1,MIN(Variables!$B$32,260)*M142+Variables!$B$31*Variables!$B$2,IF(MOD(A142-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A142-1))*M142,0))-IF(A142=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD142" s="12">
@@ -19392,7 +19407,7 @@
         <v/>
       </c>
       <c r="AC143" s="11">
-        <f>IF(MOD(A143-1,Variables!$B$30)=0,Variables!$B$30*M143,0)</f>
+        <f>IF(A143=1,MIN(Variables!$B$32,260)*M143+Variables!$B$31*Variables!$B$2,IF(MOD(A143-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A143-1))*M143,0))-IF(A143=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD143" s="12">
@@ -19517,7 +19532,7 @@
         <v/>
       </c>
       <c r="AC144" s="11">
-        <f>IF(MOD(A144-1,Variables!$B$30)=0,Variables!$B$30*M144,0)</f>
+        <f>IF(A144=1,MIN(Variables!$B$32,260)*M144+Variables!$B$31*Variables!$B$2,IF(MOD(A144-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A144-1))*M144,0))-IF(A144=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD144" s="12">
@@ -19642,7 +19657,7 @@
         <v/>
       </c>
       <c r="AC145" s="11">
-        <f>IF(MOD(A145-1,Variables!$B$30)=0,Variables!$B$30*M145,0)</f>
+        <f>IF(A145=1,MIN(Variables!$B$32,260)*M145+Variables!$B$31*Variables!$B$2,IF(MOD(A145-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A145-1))*M145,0))-IF(A145=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD145" s="12">
@@ -19767,7 +19782,7 @@
         <v/>
       </c>
       <c r="AC146" s="11">
-        <f>IF(MOD(A146-1,Variables!$B$30)=0,Variables!$B$30*M146,0)</f>
+        <f>IF(A146=1,MIN(Variables!$B$32,260)*M146+Variables!$B$31*Variables!$B$2,IF(MOD(A146-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A146-1))*M146,0))-IF(A146=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD146" s="12">
@@ -19892,7 +19907,7 @@
         <v/>
       </c>
       <c r="AC147" s="11">
-        <f>IF(MOD(A147-1,Variables!$B$30)=0,Variables!$B$30*M147,0)</f>
+        <f>IF(A147=1,MIN(Variables!$B$32,260)*M147+Variables!$B$31*Variables!$B$2,IF(MOD(A147-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A147-1))*M147,0))-IF(A147=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD147" s="12">
@@ -20017,7 +20032,7 @@
         <v/>
       </c>
       <c r="AC148" s="11">
-        <f>IF(MOD(A148-1,Variables!$B$30)=0,Variables!$B$30*M148,0)</f>
+        <f>IF(A148=1,MIN(Variables!$B$32,260)*M148+Variables!$B$31*Variables!$B$2,IF(MOD(A148-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A148-1))*M148,0))-IF(A148=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD148" s="12">
@@ -20142,7 +20157,7 @@
         <v/>
       </c>
       <c r="AC149" s="11">
-        <f>IF(MOD(A149-1,Variables!$B$30)=0,Variables!$B$30*M149,0)</f>
+        <f>IF(A149=1,MIN(Variables!$B$32,260)*M149+Variables!$B$31*Variables!$B$2,IF(MOD(A149-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A149-1))*M149,0))-IF(A149=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD149" s="12">
@@ -20267,7 +20282,7 @@
         <v/>
       </c>
       <c r="AC150" s="11">
-        <f>IF(MOD(A150-1,Variables!$B$30)=0,Variables!$B$30*M150,0)</f>
+        <f>IF(A150=1,MIN(Variables!$B$32,260)*M150+Variables!$B$31*Variables!$B$2,IF(MOD(A150-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A150-1))*M150,0))-IF(A150=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD150" s="12">
@@ -20392,7 +20407,7 @@
         <v/>
       </c>
       <c r="AC151" s="11">
-        <f>IF(MOD(A151-1,Variables!$B$30)=0,Variables!$B$30*M151,0)</f>
+        <f>IF(A151=1,MIN(Variables!$B$32,260)*M151+Variables!$B$31*Variables!$B$2,IF(MOD(A151-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A151-1))*M151,0))-IF(A151=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD151" s="12">
@@ -20517,7 +20532,7 @@
         <v/>
       </c>
       <c r="AC152" s="11">
-        <f>IF(MOD(A152-1,Variables!$B$30)=0,Variables!$B$30*M152,0)</f>
+        <f>IF(A152=1,MIN(Variables!$B$32,260)*M152+Variables!$B$31*Variables!$B$2,IF(MOD(A152-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A152-1))*M152,0))-IF(A152=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD152" s="12">
@@ -20642,7 +20657,7 @@
         <v/>
       </c>
       <c r="AC153" s="11">
-        <f>IF(MOD(A153-1,Variables!$B$30)=0,Variables!$B$30*M153,0)</f>
+        <f>IF(A153=1,MIN(Variables!$B$32,260)*M153+Variables!$B$31*Variables!$B$2,IF(MOD(A153-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A153-1))*M153,0))-IF(A153=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD153" s="12">
@@ -20767,7 +20782,7 @@
         <v/>
       </c>
       <c r="AC154" s="11">
-        <f>IF(MOD(A154-1,Variables!$B$30)=0,Variables!$B$30*M154,0)</f>
+        <f>IF(A154=1,MIN(Variables!$B$32,260)*M154+Variables!$B$31*Variables!$B$2,IF(MOD(A154-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A154-1))*M154,0))-IF(A154=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD154" s="12">
@@ -20892,7 +20907,7 @@
         <v/>
       </c>
       <c r="AC155" s="11">
-        <f>IF(MOD(A155-1,Variables!$B$30)=0,Variables!$B$30*M155,0)</f>
+        <f>IF(A155=1,MIN(Variables!$B$32,260)*M155+Variables!$B$31*Variables!$B$2,IF(MOD(A155-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A155-1))*M155,0))-IF(A155=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD155" s="12">
@@ -21017,7 +21032,7 @@
         <v/>
       </c>
       <c r="AC156" s="11">
-        <f>IF(MOD(A156-1,Variables!$B$30)=0,Variables!$B$30*M156,0)</f>
+        <f>IF(A156=1,MIN(Variables!$B$32,260)*M156+Variables!$B$31*Variables!$B$2,IF(MOD(A156-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A156-1))*M156,0))-IF(A156=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD156" s="12">
@@ -21142,7 +21157,7 @@
         <v/>
       </c>
       <c r="AC157" s="11">
-        <f>IF(MOD(A157-1,Variables!$B$30)=0,Variables!$B$30*M157,0)</f>
+        <f>IF(A157=1,MIN(Variables!$B$32,260)*M157+Variables!$B$31*Variables!$B$2,IF(MOD(A157-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A157-1))*M157,0))-IF(A157=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD157" s="12">
@@ -21267,7 +21282,7 @@
         <v/>
       </c>
       <c r="AC158" s="11">
-        <f>IF(MOD(A158-1,Variables!$B$30)=0,Variables!$B$30*M158,0)</f>
+        <f>IF(A158=1,MIN(Variables!$B$32,260)*M158+Variables!$B$31*Variables!$B$2,IF(MOD(A158-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A158-1))*M158,0))-IF(A158=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD158" s="12">
@@ -21392,7 +21407,7 @@
         <v/>
       </c>
       <c r="AC159" s="11">
-        <f>IF(MOD(A159-1,Variables!$B$30)=0,Variables!$B$30*M159,0)</f>
+        <f>IF(A159=1,MIN(Variables!$B$32,260)*M159+Variables!$B$31*Variables!$B$2,IF(MOD(A159-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A159-1))*M159,0))-IF(A159=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD159" s="12">
@@ -21517,7 +21532,7 @@
         <v/>
       </c>
       <c r="AC160" s="11">
-        <f>IF(MOD(A160-1,Variables!$B$30)=0,Variables!$B$30*M160,0)</f>
+        <f>IF(A160=1,MIN(Variables!$B$32,260)*M160+Variables!$B$31*Variables!$B$2,IF(MOD(A160-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A160-1))*M160,0))-IF(A160=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD160" s="12">
@@ -21642,7 +21657,7 @@
         <v/>
       </c>
       <c r="AC161" s="11">
-        <f>IF(MOD(A161-1,Variables!$B$30)=0,Variables!$B$30*M161,0)</f>
+        <f>IF(A161=1,MIN(Variables!$B$32,260)*M161+Variables!$B$31*Variables!$B$2,IF(MOD(A161-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A161-1))*M161,0))-IF(A161=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD161" s="12">
@@ -21767,7 +21782,7 @@
         <v/>
       </c>
       <c r="AC162" s="11">
-        <f>IF(MOD(A162-1,Variables!$B$30)=0,Variables!$B$30*M162,0)</f>
+        <f>IF(A162=1,MIN(Variables!$B$32,260)*M162+Variables!$B$31*Variables!$B$2,IF(MOD(A162-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A162-1))*M162,0))-IF(A162=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD162" s="12">
@@ -21892,7 +21907,7 @@
         <v/>
       </c>
       <c r="AC163" s="11">
-        <f>IF(MOD(A163-1,Variables!$B$30)=0,Variables!$B$30*M163,0)</f>
+        <f>IF(A163=1,MIN(Variables!$B$32,260)*M163+Variables!$B$31*Variables!$B$2,IF(MOD(A163-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A163-1))*M163,0))-IF(A163=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD163" s="12">
@@ -22017,7 +22032,7 @@
         <v/>
       </c>
       <c r="AC164" s="11">
-        <f>IF(MOD(A164-1,Variables!$B$30)=0,Variables!$B$30*M164,0)</f>
+        <f>IF(A164=1,MIN(Variables!$B$32,260)*M164+Variables!$B$31*Variables!$B$2,IF(MOD(A164-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A164-1))*M164,0))-IF(A164=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD164" s="12">
@@ -22142,7 +22157,7 @@
         <v/>
       </c>
       <c r="AC165" s="11">
-        <f>IF(MOD(A165-1,Variables!$B$30)=0,Variables!$B$30*M165,0)</f>
+        <f>IF(A165=1,MIN(Variables!$B$32,260)*M165+Variables!$B$31*Variables!$B$2,IF(MOD(A165-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A165-1))*M165,0))-IF(A165=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD165" s="12">
@@ -22267,7 +22282,7 @@
         <v/>
       </c>
       <c r="AC166" s="11">
-        <f>IF(MOD(A166-1,Variables!$B$30)=0,Variables!$B$30*M166,0)</f>
+        <f>IF(A166=1,MIN(Variables!$B$32,260)*M166+Variables!$B$31*Variables!$B$2,IF(MOD(A166-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A166-1))*M166,0))-IF(A166=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD166" s="12">
@@ -22392,7 +22407,7 @@
         <v/>
       </c>
       <c r="AC167" s="11">
-        <f>IF(MOD(A167-1,Variables!$B$30)=0,Variables!$B$30*M167,0)</f>
+        <f>IF(A167=1,MIN(Variables!$B$32,260)*M167+Variables!$B$31*Variables!$B$2,IF(MOD(A167-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A167-1))*M167,0))-IF(A167=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD167" s="12">
@@ -22517,7 +22532,7 @@
         <v/>
       </c>
       <c r="AC168" s="11">
-        <f>IF(MOD(A168-1,Variables!$B$30)=0,Variables!$B$30*M168,0)</f>
+        <f>IF(A168=1,MIN(Variables!$B$32,260)*M168+Variables!$B$31*Variables!$B$2,IF(MOD(A168-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A168-1))*M168,0))-IF(A168=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD168" s="12">
@@ -22642,7 +22657,7 @@
         <v/>
       </c>
       <c r="AC169" s="11">
-        <f>IF(MOD(A169-1,Variables!$B$30)=0,Variables!$B$30*M169,0)</f>
+        <f>IF(A169=1,MIN(Variables!$B$32,260)*M169+Variables!$B$31*Variables!$B$2,IF(MOD(A169-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A169-1))*M169,0))-IF(A169=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD169" s="12">
@@ -22767,7 +22782,7 @@
         <v/>
       </c>
       <c r="AC170" s="11">
-        <f>IF(MOD(A170-1,Variables!$B$30)=0,Variables!$B$30*M170,0)</f>
+        <f>IF(A170=1,MIN(Variables!$B$32,260)*M170+Variables!$B$31*Variables!$B$2,IF(MOD(A170-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A170-1))*M170,0))-IF(A170=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD170" s="12">
@@ -22892,7 +22907,7 @@
         <v/>
       </c>
       <c r="AC171" s="11">
-        <f>IF(MOD(A171-1,Variables!$B$30)=0,Variables!$B$30*M171,0)</f>
+        <f>IF(A171=1,MIN(Variables!$B$32,260)*M171+Variables!$B$31*Variables!$B$2,IF(MOD(A171-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A171-1))*M171,0))-IF(A171=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD171" s="12">
@@ -23017,7 +23032,7 @@
         <v/>
       </c>
       <c r="AC172" s="11">
-        <f>IF(MOD(A172-1,Variables!$B$30)=0,Variables!$B$30*M172,0)</f>
+        <f>IF(A172=1,MIN(Variables!$B$32,260)*M172+Variables!$B$31*Variables!$B$2,IF(MOD(A172-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A172-1))*M172,0))-IF(A172=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD172" s="12">
@@ -23142,7 +23157,7 @@
         <v/>
       </c>
       <c r="AC173" s="11">
-        <f>IF(MOD(A173-1,Variables!$B$30)=0,Variables!$B$30*M173,0)</f>
+        <f>IF(A173=1,MIN(Variables!$B$32,260)*M173+Variables!$B$31*Variables!$B$2,IF(MOD(A173-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A173-1))*M173,0))-IF(A173=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD173" s="12">
@@ -23267,7 +23282,7 @@
         <v/>
       </c>
       <c r="AC174" s="11">
-        <f>IF(MOD(A174-1,Variables!$B$30)=0,Variables!$B$30*M174,0)</f>
+        <f>IF(A174=1,MIN(Variables!$B$32,260)*M174+Variables!$B$31*Variables!$B$2,IF(MOD(A174-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A174-1))*M174,0))-IF(A174=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD174" s="12">
@@ -23392,7 +23407,7 @@
         <v/>
       </c>
       <c r="AC175" s="11">
-        <f>IF(MOD(A175-1,Variables!$B$30)=0,Variables!$B$30*M175,0)</f>
+        <f>IF(A175=1,MIN(Variables!$B$32,260)*M175+Variables!$B$31*Variables!$B$2,IF(MOD(A175-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A175-1))*M175,0))-IF(A175=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD175" s="12">
@@ -23517,7 +23532,7 @@
         <v/>
       </c>
       <c r="AC176" s="11">
-        <f>IF(MOD(A176-1,Variables!$B$30)=0,Variables!$B$30*M176,0)</f>
+        <f>IF(A176=1,MIN(Variables!$B$32,260)*M176+Variables!$B$31*Variables!$B$2,IF(MOD(A176-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A176-1))*M176,0))-IF(A176=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD176" s="12">
@@ -23642,7 +23657,7 @@
         <v/>
       </c>
       <c r="AC177" s="11">
-        <f>IF(MOD(A177-1,Variables!$B$30)=0,Variables!$B$30*M177,0)</f>
+        <f>IF(A177=1,MIN(Variables!$B$32,260)*M177+Variables!$B$31*Variables!$B$2,IF(MOD(A177-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A177-1))*M177,0))-IF(A177=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD177" s="12">
@@ -23767,7 +23782,7 @@
         <v/>
       </c>
       <c r="AC178" s="11">
-        <f>IF(MOD(A178-1,Variables!$B$30)=0,Variables!$B$30*M178,0)</f>
+        <f>IF(A178=1,MIN(Variables!$B$32,260)*M178+Variables!$B$31*Variables!$B$2,IF(MOD(A178-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A178-1))*M178,0))-IF(A178=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD178" s="12">
@@ -23892,7 +23907,7 @@
         <v/>
       </c>
       <c r="AC179" s="11">
-        <f>IF(MOD(A179-1,Variables!$B$30)=0,Variables!$B$30*M179,0)</f>
+        <f>IF(A179=1,MIN(Variables!$B$32,260)*M179+Variables!$B$31*Variables!$B$2,IF(MOD(A179-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A179-1))*M179,0))-IF(A179=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD179" s="12">
@@ -24017,7 +24032,7 @@
         <v/>
       </c>
       <c r="AC180" s="11">
-        <f>IF(MOD(A180-1,Variables!$B$30)=0,Variables!$B$30*M180,0)</f>
+        <f>IF(A180=1,MIN(Variables!$B$32,260)*M180+Variables!$B$31*Variables!$B$2,IF(MOD(A180-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A180-1))*M180,0))-IF(A180=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD180" s="12">
@@ -24142,7 +24157,7 @@
         <v/>
       </c>
       <c r="AC181" s="11">
-        <f>IF(MOD(A181-1,Variables!$B$30)=0,Variables!$B$30*M181,0)</f>
+        <f>IF(A181=1,MIN(Variables!$B$32,260)*M181+Variables!$B$31*Variables!$B$2,IF(MOD(A181-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A181-1))*M181,0))-IF(A181=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD181" s="12">
@@ -24267,7 +24282,7 @@
         <v/>
       </c>
       <c r="AC182" s="11">
-        <f>IF(MOD(A182-1,Variables!$B$30)=0,Variables!$B$30*M182,0)</f>
+        <f>IF(A182=1,MIN(Variables!$B$32,260)*M182+Variables!$B$31*Variables!$B$2,IF(MOD(A182-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A182-1))*M182,0))-IF(A182=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD182" s="12">
@@ -24392,7 +24407,7 @@
         <v/>
       </c>
       <c r="AC183" s="11">
-        <f>IF(MOD(A183-1,Variables!$B$30)=0,Variables!$B$30*M183,0)</f>
+        <f>IF(A183=1,MIN(Variables!$B$32,260)*M183+Variables!$B$31*Variables!$B$2,IF(MOD(A183-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A183-1))*M183,0))-IF(A183=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD183" s="12">
@@ -24517,7 +24532,7 @@
         <v/>
       </c>
       <c r="AC184" s="11">
-        <f>IF(MOD(A184-1,Variables!$B$30)=0,Variables!$B$30*M184,0)</f>
+        <f>IF(A184=1,MIN(Variables!$B$32,260)*M184+Variables!$B$31*Variables!$B$2,IF(MOD(A184-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A184-1))*M184,0))-IF(A184=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD184" s="12">
@@ -24642,7 +24657,7 @@
         <v/>
       </c>
       <c r="AC185" s="11">
-        <f>IF(MOD(A185-1,Variables!$B$30)=0,Variables!$B$30*M185,0)</f>
+        <f>IF(A185=1,MIN(Variables!$B$32,260)*M185+Variables!$B$31*Variables!$B$2,IF(MOD(A185-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A185-1))*M185,0))-IF(A185=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD185" s="12">
@@ -24767,7 +24782,7 @@
         <v/>
       </c>
       <c r="AC186" s="11">
-        <f>IF(MOD(A186-1,Variables!$B$30)=0,Variables!$B$30*M186,0)</f>
+        <f>IF(A186=1,MIN(Variables!$B$32,260)*M186+Variables!$B$31*Variables!$B$2,IF(MOD(A186-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A186-1))*M186,0))-IF(A186=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD186" s="12">
@@ -24892,7 +24907,7 @@
         <v/>
       </c>
       <c r="AC187" s="11">
-        <f>IF(MOD(A187-1,Variables!$B$30)=0,Variables!$B$30*M187,0)</f>
+        <f>IF(A187=1,MIN(Variables!$B$32,260)*M187+Variables!$B$31*Variables!$B$2,IF(MOD(A187-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A187-1))*M187,0))-IF(A187=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD187" s="12">
@@ -25017,7 +25032,7 @@
         <v/>
       </c>
       <c r="AC188" s="11">
-        <f>IF(MOD(A188-1,Variables!$B$30)=0,Variables!$B$30*M188,0)</f>
+        <f>IF(A188=1,MIN(Variables!$B$32,260)*M188+Variables!$B$31*Variables!$B$2,IF(MOD(A188-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A188-1))*M188,0))-IF(A188=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD188" s="12">
@@ -25142,7 +25157,7 @@
         <v/>
       </c>
       <c r="AC189" s="11">
-        <f>IF(MOD(A189-1,Variables!$B$30)=0,Variables!$B$30*M189,0)</f>
+        <f>IF(A189=1,MIN(Variables!$B$32,260)*M189+Variables!$B$31*Variables!$B$2,IF(MOD(A189-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A189-1))*M189,0))-IF(A189=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD189" s="12">
@@ -25267,7 +25282,7 @@
         <v/>
       </c>
       <c r="AC190" s="11">
-        <f>IF(MOD(A190-1,Variables!$B$30)=0,Variables!$B$30*M190,0)</f>
+        <f>IF(A190=1,MIN(Variables!$B$32,260)*M190+Variables!$B$31*Variables!$B$2,IF(MOD(A190-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A190-1))*M190,0))-IF(A190=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD190" s="12">
@@ -25392,7 +25407,7 @@
         <v/>
       </c>
       <c r="AC191" s="11">
-        <f>IF(MOD(A191-1,Variables!$B$30)=0,Variables!$B$30*M191,0)</f>
+        <f>IF(A191=1,MIN(Variables!$B$32,260)*M191+Variables!$B$31*Variables!$B$2,IF(MOD(A191-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A191-1))*M191,0))-IF(A191=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD191" s="12">
@@ -25517,7 +25532,7 @@
         <v/>
       </c>
       <c r="AC192" s="11">
-        <f>IF(MOD(A192-1,Variables!$B$30)=0,Variables!$B$30*M192,0)</f>
+        <f>IF(A192=1,MIN(Variables!$B$32,260)*M192+Variables!$B$31*Variables!$B$2,IF(MOD(A192-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A192-1))*M192,0))-IF(A192=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD192" s="12">
@@ -25642,7 +25657,7 @@
         <v/>
       </c>
       <c r="AC193" s="11">
-        <f>IF(MOD(A193-1,Variables!$B$30)=0,Variables!$B$30*M193,0)</f>
+        <f>IF(A193=1,MIN(Variables!$B$32,260)*M193+Variables!$B$31*Variables!$B$2,IF(MOD(A193-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A193-1))*M193,0))-IF(A193=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD193" s="12">
@@ -25767,7 +25782,7 @@
         <v/>
       </c>
       <c r="AC194" s="11">
-        <f>IF(MOD(A194-1,Variables!$B$30)=0,Variables!$B$30*M194,0)</f>
+        <f>IF(A194=1,MIN(Variables!$B$32,260)*M194+Variables!$B$31*Variables!$B$2,IF(MOD(A194-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A194-1))*M194,0))-IF(A194=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD194" s="12">
@@ -25892,7 +25907,7 @@
         <v/>
       </c>
       <c r="AC195" s="11">
-        <f>IF(MOD(A195-1,Variables!$B$30)=0,Variables!$B$30*M195,0)</f>
+        <f>IF(A195=1,MIN(Variables!$B$32,260)*M195+Variables!$B$31*Variables!$B$2,IF(MOD(A195-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A195-1))*M195,0))-IF(A195=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD195" s="12">
@@ -26017,7 +26032,7 @@
         <v/>
       </c>
       <c r="AC196" s="11">
-        <f>IF(MOD(A196-1,Variables!$B$30)=0,Variables!$B$30*M196,0)</f>
+        <f>IF(A196=1,MIN(Variables!$B$32,260)*M196+Variables!$B$31*Variables!$B$2,IF(MOD(A196-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A196-1))*M196,0))-IF(A196=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD196" s="12">
@@ -26142,7 +26157,7 @@
         <v/>
       </c>
       <c r="AC197" s="11">
-        <f>IF(MOD(A197-1,Variables!$B$30)=0,Variables!$B$30*M197,0)</f>
+        <f>IF(A197=1,MIN(Variables!$B$32,260)*M197+Variables!$B$31*Variables!$B$2,IF(MOD(A197-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A197-1))*M197,0))-IF(A197=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD197" s="12">
@@ -26267,7 +26282,7 @@
         <v/>
       </c>
       <c r="AC198" s="11">
-        <f>IF(MOD(A198-1,Variables!$B$30)=0,Variables!$B$30*M198,0)</f>
+        <f>IF(A198=1,MIN(Variables!$B$32,260)*M198+Variables!$B$31*Variables!$B$2,IF(MOD(A198-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A198-1))*M198,0))-IF(A198=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD198" s="12">
@@ -26392,7 +26407,7 @@
         <v/>
       </c>
       <c r="AC199" s="11">
-        <f>IF(MOD(A199-1,Variables!$B$30)=0,Variables!$B$30*M199,0)</f>
+        <f>IF(A199=1,MIN(Variables!$B$32,260)*M199+Variables!$B$31*Variables!$B$2,IF(MOD(A199-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A199-1))*M199,0))-IF(A199=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD199" s="12">
@@ -26517,7 +26532,7 @@
         <v/>
       </c>
       <c r="AC200" s="11">
-        <f>IF(MOD(A200-1,Variables!$B$30)=0,Variables!$B$30*M200,0)</f>
+        <f>IF(A200=1,MIN(Variables!$B$32,260)*M200+Variables!$B$31*Variables!$B$2,IF(MOD(A200-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A200-1))*M200,0))-IF(A200=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD200" s="12">
@@ -26642,7 +26657,7 @@
         <v/>
       </c>
       <c r="AC201" s="11">
-        <f>IF(MOD(A201-1,Variables!$B$30)=0,Variables!$B$30*M201,0)</f>
+        <f>IF(A201=1,MIN(Variables!$B$32,260)*M201+Variables!$B$31*Variables!$B$2,IF(MOD(A201-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A201-1))*M201,0))-IF(A201=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD201" s="12">
@@ -26767,7 +26782,7 @@
         <v/>
       </c>
       <c r="AC202" s="11">
-        <f>IF(MOD(A202-1,Variables!$B$30)=0,Variables!$B$30*M202,0)</f>
+        <f>IF(A202=1,MIN(Variables!$B$32,260)*M202+Variables!$B$31*Variables!$B$2,IF(MOD(A202-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A202-1))*M202,0))-IF(A202=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD202" s="12">
@@ -26892,7 +26907,7 @@
         <v/>
       </c>
       <c r="AC203" s="11">
-        <f>IF(MOD(A203-1,Variables!$B$30)=0,Variables!$B$30*M203,0)</f>
+        <f>IF(A203=1,MIN(Variables!$B$32,260)*M203+Variables!$B$31*Variables!$B$2,IF(MOD(A203-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A203-1))*M203,0))-IF(A203=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD203" s="12">
@@ -27017,7 +27032,7 @@
         <v/>
       </c>
       <c r="AC204" s="11">
-        <f>IF(MOD(A204-1,Variables!$B$30)=0,Variables!$B$30*M204,0)</f>
+        <f>IF(A204=1,MIN(Variables!$B$32,260)*M204+Variables!$B$31*Variables!$B$2,IF(MOD(A204-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A204-1))*M204,0))-IF(A204=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD204" s="12">
@@ -27142,7 +27157,7 @@
         <v/>
       </c>
       <c r="AC205" s="11">
-        <f>IF(MOD(A205-1,Variables!$B$30)=0,Variables!$B$30*M205,0)</f>
+        <f>IF(A205=1,MIN(Variables!$B$32,260)*M205+Variables!$B$31*Variables!$B$2,IF(MOD(A205-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A205-1))*M205,0))-IF(A205=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD205" s="12">
@@ -27267,7 +27282,7 @@
         <v/>
       </c>
       <c r="AC206" s="11">
-        <f>IF(MOD(A206-1,Variables!$B$30)=0,Variables!$B$30*M206,0)</f>
+        <f>IF(A206=1,MIN(Variables!$B$32,260)*M206+Variables!$B$31*Variables!$B$2,IF(MOD(A206-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A206-1))*M206,0))-IF(A206=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD206" s="12">
@@ -27392,7 +27407,7 @@
         <v/>
       </c>
       <c r="AC207" s="11">
-        <f>IF(MOD(A207-1,Variables!$B$30)=0,Variables!$B$30*M207,0)</f>
+        <f>IF(A207=1,MIN(Variables!$B$32,260)*M207+Variables!$B$31*Variables!$B$2,IF(MOD(A207-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A207-1))*M207,0))-IF(A207=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD207" s="12">
@@ -27517,7 +27532,7 @@
         <v/>
       </c>
       <c r="AC208" s="11">
-        <f>IF(MOD(A208-1,Variables!$B$30)=0,Variables!$B$30*M208,0)</f>
+        <f>IF(A208=1,MIN(Variables!$B$32,260)*M208+Variables!$B$31*Variables!$B$2,IF(MOD(A208-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A208-1))*M208,0))-IF(A208=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD208" s="12">
@@ -27642,7 +27657,7 @@
         <v/>
       </c>
       <c r="AC209" s="11">
-        <f>IF(MOD(A209-1,Variables!$B$30)=0,Variables!$B$30*M209,0)</f>
+        <f>IF(A209=1,MIN(Variables!$B$32,260)*M209+Variables!$B$31*Variables!$B$2,IF(MOD(A209-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A209-1))*M209,0))-IF(A209=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD209" s="12">
@@ -27767,7 +27782,7 @@
         <v/>
       </c>
       <c r="AC210" s="11">
-        <f>IF(MOD(A210-1,Variables!$B$30)=0,Variables!$B$30*M210,0)</f>
+        <f>IF(A210=1,MIN(Variables!$B$32,260)*M210+Variables!$B$31*Variables!$B$2,IF(MOD(A210-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A210-1))*M210,0))-IF(A210=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD210" s="12">
@@ -27892,7 +27907,7 @@
         <v/>
       </c>
       <c r="AC211" s="11">
-        <f>IF(MOD(A211-1,Variables!$B$30)=0,Variables!$B$30*M211,0)</f>
+        <f>IF(A211=1,MIN(Variables!$B$32,260)*M211+Variables!$B$31*Variables!$B$2,IF(MOD(A211-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A211-1))*M211,0))-IF(A211=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD211" s="12">
@@ -28017,7 +28032,7 @@
         <v/>
       </c>
       <c r="AC212" s="11">
-        <f>IF(MOD(A212-1,Variables!$B$30)=0,Variables!$B$30*M212,0)</f>
+        <f>IF(A212=1,MIN(Variables!$B$32,260)*M212+Variables!$B$31*Variables!$B$2,IF(MOD(A212-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A212-1))*M212,0))-IF(A212=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD212" s="12">
@@ -28142,7 +28157,7 @@
         <v/>
       </c>
       <c r="AC213" s="11">
-        <f>IF(MOD(A213-1,Variables!$B$30)=0,Variables!$B$30*M213,0)</f>
+        <f>IF(A213=1,MIN(Variables!$B$32,260)*M213+Variables!$B$31*Variables!$B$2,IF(MOD(A213-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A213-1))*M213,0))-IF(A213=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD213" s="12">
@@ -28267,7 +28282,7 @@
         <v/>
       </c>
       <c r="AC214" s="11">
-        <f>IF(MOD(A214-1,Variables!$B$30)=0,Variables!$B$30*M214,0)</f>
+        <f>IF(A214=1,MIN(Variables!$B$32,260)*M214+Variables!$B$31*Variables!$B$2,IF(MOD(A214-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A214-1))*M214,0))-IF(A214=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD214" s="12">
@@ -28392,7 +28407,7 @@
         <v/>
       </c>
       <c r="AC215" s="11">
-        <f>IF(MOD(A215-1,Variables!$B$30)=0,Variables!$B$30*M215,0)</f>
+        <f>IF(A215=1,MIN(Variables!$B$32,260)*M215+Variables!$B$31*Variables!$B$2,IF(MOD(A215-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A215-1))*M215,0))-IF(A215=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD215" s="12">
@@ -28517,7 +28532,7 @@
         <v/>
       </c>
       <c r="AC216" s="11">
-        <f>IF(MOD(A216-1,Variables!$B$30)=0,Variables!$B$30*M216,0)</f>
+        <f>IF(A216=1,MIN(Variables!$B$32,260)*M216+Variables!$B$31*Variables!$B$2,IF(MOD(A216-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A216-1))*M216,0))-IF(A216=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD216" s="12">
@@ -28642,7 +28657,7 @@
         <v/>
       </c>
       <c r="AC217" s="11">
-        <f>IF(MOD(A217-1,Variables!$B$30)=0,Variables!$B$30*M217,0)</f>
+        <f>IF(A217=1,MIN(Variables!$B$32,260)*M217+Variables!$B$31*Variables!$B$2,IF(MOD(A217-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A217-1))*M217,0))-IF(A217=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD217" s="12">
@@ -28767,7 +28782,7 @@
         <v/>
       </c>
       <c r="AC218" s="11">
-        <f>IF(MOD(A218-1,Variables!$B$30)=0,Variables!$B$30*M218,0)</f>
+        <f>IF(A218=1,MIN(Variables!$B$32,260)*M218+Variables!$B$31*Variables!$B$2,IF(MOD(A218-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A218-1))*M218,0))-IF(A218=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD218" s="12">
@@ -28892,7 +28907,7 @@
         <v/>
       </c>
       <c r="AC219" s="11">
-        <f>IF(MOD(A219-1,Variables!$B$30)=0,Variables!$B$30*M219,0)</f>
+        <f>IF(A219=1,MIN(Variables!$B$32,260)*M219+Variables!$B$31*Variables!$B$2,IF(MOD(A219-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A219-1))*M219,0))-IF(A219=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD219" s="12">
@@ -29017,7 +29032,7 @@
         <v/>
       </c>
       <c r="AC220" s="11">
-        <f>IF(MOD(A220-1,Variables!$B$30)=0,Variables!$B$30*M220,0)</f>
+        <f>IF(A220=1,MIN(Variables!$B$32,260)*M220+Variables!$B$31*Variables!$B$2,IF(MOD(A220-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A220-1))*M220,0))-IF(A220=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD220" s="12">
@@ -29142,7 +29157,7 @@
         <v/>
       </c>
       <c r="AC221" s="11">
-        <f>IF(MOD(A221-1,Variables!$B$30)=0,Variables!$B$30*M221,0)</f>
+        <f>IF(A221=1,MIN(Variables!$B$32,260)*M221+Variables!$B$31*Variables!$B$2,IF(MOD(A221-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A221-1))*M221,0))-IF(A221=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD221" s="12">
@@ -29267,7 +29282,7 @@
         <v/>
       </c>
       <c r="AC222" s="11">
-        <f>IF(MOD(A222-1,Variables!$B$30)=0,Variables!$B$30*M222,0)</f>
+        <f>IF(A222=1,MIN(Variables!$B$32,260)*M222+Variables!$B$31*Variables!$B$2,IF(MOD(A222-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A222-1))*M222,0))-IF(A222=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD222" s="12">
@@ -29392,7 +29407,7 @@
         <v/>
       </c>
       <c r="AC223" s="11">
-        <f>IF(MOD(A223-1,Variables!$B$30)=0,Variables!$B$30*M223,0)</f>
+        <f>IF(A223=1,MIN(Variables!$B$32,260)*M223+Variables!$B$31*Variables!$B$2,IF(MOD(A223-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A223-1))*M223,0))-IF(A223=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD223" s="12">
@@ -29517,7 +29532,7 @@
         <v/>
       </c>
       <c r="AC224" s="11">
-        <f>IF(MOD(A224-1,Variables!$B$30)=0,Variables!$B$30*M224,0)</f>
+        <f>IF(A224=1,MIN(Variables!$B$32,260)*M224+Variables!$B$31*Variables!$B$2,IF(MOD(A224-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A224-1))*M224,0))-IF(A224=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD224" s="12">
@@ -29642,7 +29657,7 @@
         <v/>
       </c>
       <c r="AC225" s="11">
-        <f>IF(MOD(A225-1,Variables!$B$30)=0,Variables!$B$30*M225,0)</f>
+        <f>IF(A225=1,MIN(Variables!$B$32,260)*M225+Variables!$B$31*Variables!$B$2,IF(MOD(A225-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A225-1))*M225,0))-IF(A225=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD225" s="12">
@@ -29767,7 +29782,7 @@
         <v/>
       </c>
       <c r="AC226" s="11">
-        <f>IF(MOD(A226-1,Variables!$B$30)=0,Variables!$B$30*M226,0)</f>
+        <f>IF(A226=1,MIN(Variables!$B$32,260)*M226+Variables!$B$31*Variables!$B$2,IF(MOD(A226-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A226-1))*M226,0))-IF(A226=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD226" s="12">
@@ -29892,7 +29907,7 @@
         <v/>
       </c>
       <c r="AC227" s="11">
-        <f>IF(MOD(A227-1,Variables!$B$30)=0,Variables!$B$30*M227,0)</f>
+        <f>IF(A227=1,MIN(Variables!$B$32,260)*M227+Variables!$B$31*Variables!$B$2,IF(MOD(A227-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A227-1))*M227,0))-IF(A227=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD227" s="12">
@@ -30017,7 +30032,7 @@
         <v/>
       </c>
       <c r="AC228" s="11">
-        <f>IF(MOD(A228-1,Variables!$B$30)=0,Variables!$B$30*M228,0)</f>
+        <f>IF(A228=1,MIN(Variables!$B$32,260)*M228+Variables!$B$31*Variables!$B$2,IF(MOD(A228-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A228-1))*M228,0))-IF(A228=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD228" s="12">
@@ -30142,7 +30157,7 @@
         <v/>
       </c>
       <c r="AC229" s="11">
-        <f>IF(MOD(A229-1,Variables!$B$30)=0,Variables!$B$30*M229,0)</f>
+        <f>IF(A229=1,MIN(Variables!$B$32,260)*M229+Variables!$B$31*Variables!$B$2,IF(MOD(A229-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A229-1))*M229,0))-IF(A229=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD229" s="12">
@@ -30267,7 +30282,7 @@
         <v/>
       </c>
       <c r="AC230" s="11">
-        <f>IF(MOD(A230-1,Variables!$B$30)=0,Variables!$B$30*M230,0)</f>
+        <f>IF(A230=1,MIN(Variables!$B$32,260)*M230+Variables!$B$31*Variables!$B$2,IF(MOD(A230-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A230-1))*M230,0))-IF(A230=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD230" s="12">
@@ -30392,7 +30407,7 @@
         <v/>
       </c>
       <c r="AC231" s="11">
-        <f>IF(MOD(A231-1,Variables!$B$30)=0,Variables!$B$30*M231,0)</f>
+        <f>IF(A231=1,MIN(Variables!$B$32,260)*M231+Variables!$B$31*Variables!$B$2,IF(MOD(A231-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A231-1))*M231,0))-IF(A231=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD231" s="12">
@@ -30517,7 +30532,7 @@
         <v/>
       </c>
       <c r="AC232" s="11">
-        <f>IF(MOD(A232-1,Variables!$B$30)=0,Variables!$B$30*M232,0)</f>
+        <f>IF(A232=1,MIN(Variables!$B$32,260)*M232+Variables!$B$31*Variables!$B$2,IF(MOD(A232-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A232-1))*M232,0))-IF(A232=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD232" s="12">
@@ -30642,7 +30657,7 @@
         <v/>
       </c>
       <c r="AC233" s="11">
-        <f>IF(MOD(A233-1,Variables!$B$30)=0,Variables!$B$30*M233,0)</f>
+        <f>IF(A233=1,MIN(Variables!$B$32,260)*M233+Variables!$B$31*Variables!$B$2,IF(MOD(A233-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A233-1))*M233,0))-IF(A233=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD233" s="12">
@@ -30767,7 +30782,7 @@
         <v/>
       </c>
       <c r="AC234" s="11">
-        <f>IF(MOD(A234-1,Variables!$B$30)=0,Variables!$B$30*M234,0)</f>
+        <f>IF(A234=1,MIN(Variables!$B$32,260)*M234+Variables!$B$31*Variables!$B$2,IF(MOD(A234-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A234-1))*M234,0))-IF(A234=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD234" s="12">
@@ -30892,7 +30907,7 @@
         <v/>
       </c>
       <c r="AC235" s="11">
-        <f>IF(MOD(A235-1,Variables!$B$30)=0,Variables!$B$30*M235,0)</f>
+        <f>IF(A235=1,MIN(Variables!$B$32,260)*M235+Variables!$B$31*Variables!$B$2,IF(MOD(A235-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A235-1))*M235,0))-IF(A235=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD235" s="12">
@@ -31017,7 +31032,7 @@
         <v/>
       </c>
       <c r="AC236" s="11">
-        <f>IF(MOD(A236-1,Variables!$B$30)=0,Variables!$B$30*M236,0)</f>
+        <f>IF(A236=1,MIN(Variables!$B$32,260)*M236+Variables!$B$31*Variables!$B$2,IF(MOD(A236-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A236-1))*M236,0))-IF(A236=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD236" s="12">
@@ -31142,7 +31157,7 @@
         <v/>
       </c>
       <c r="AC237" s="11">
-        <f>IF(MOD(A237-1,Variables!$B$30)=0,Variables!$B$30*M237,0)</f>
+        <f>IF(A237=1,MIN(Variables!$B$32,260)*M237+Variables!$B$31*Variables!$B$2,IF(MOD(A237-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A237-1))*M237,0))-IF(A237=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD237" s="12">
@@ -31267,7 +31282,7 @@
         <v/>
       </c>
       <c r="AC238" s="11">
-        <f>IF(MOD(A238-1,Variables!$B$30)=0,Variables!$B$30*M238,0)</f>
+        <f>IF(A238=1,MIN(Variables!$B$32,260)*M238+Variables!$B$31*Variables!$B$2,IF(MOD(A238-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A238-1))*M238,0))-IF(A238=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD238" s="12">
@@ -31392,7 +31407,7 @@
         <v/>
       </c>
       <c r="AC239" s="11">
-        <f>IF(MOD(A239-1,Variables!$B$30)=0,Variables!$B$30*M239,0)</f>
+        <f>IF(A239=1,MIN(Variables!$B$32,260)*M239+Variables!$B$31*Variables!$B$2,IF(MOD(A239-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A239-1))*M239,0))-IF(A239=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD239" s="12">
@@ -31517,7 +31532,7 @@
         <v/>
       </c>
       <c r="AC240" s="11">
-        <f>IF(MOD(A240-1,Variables!$B$30)=0,Variables!$B$30*M240,0)</f>
+        <f>IF(A240=1,MIN(Variables!$B$32,260)*M240+Variables!$B$31*Variables!$B$2,IF(MOD(A240-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A240-1))*M240,0))-IF(A240=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD240" s="12">
@@ -31642,7 +31657,7 @@
         <v/>
       </c>
       <c r="AC241" s="11">
-        <f>IF(MOD(A241-1,Variables!$B$30)=0,Variables!$B$30*M241,0)</f>
+        <f>IF(A241=1,MIN(Variables!$B$32,260)*M241+Variables!$B$31*Variables!$B$2,IF(MOD(A241-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A241-1))*M241,0))-IF(A241=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD241" s="12">
@@ -31767,7 +31782,7 @@
         <v/>
       </c>
       <c r="AC242" s="11">
-        <f>IF(MOD(A242-1,Variables!$B$30)=0,Variables!$B$30*M242,0)</f>
+        <f>IF(A242=1,MIN(Variables!$B$32,260)*M242+Variables!$B$31*Variables!$B$2,IF(MOD(A242-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A242-1))*M242,0))-IF(A242=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD242" s="12">
@@ -31892,7 +31907,7 @@
         <v/>
       </c>
       <c r="AC243" s="11">
-        <f>IF(MOD(A243-1,Variables!$B$30)=0,Variables!$B$30*M243,0)</f>
+        <f>IF(A243=1,MIN(Variables!$B$32,260)*M243+Variables!$B$31*Variables!$B$2,IF(MOD(A243-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A243-1))*M243,0))-IF(A243=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD243" s="12">
@@ -32017,7 +32032,7 @@
         <v/>
       </c>
       <c r="AC244" s="11">
-        <f>IF(MOD(A244-1,Variables!$B$30)=0,Variables!$B$30*M244,0)</f>
+        <f>IF(A244=1,MIN(Variables!$B$32,260)*M244+Variables!$B$31*Variables!$B$2,IF(MOD(A244-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A244-1))*M244,0))-IF(A244=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD244" s="12">
@@ -32142,7 +32157,7 @@
         <v/>
       </c>
       <c r="AC245" s="11">
-        <f>IF(MOD(A245-1,Variables!$B$30)=0,Variables!$B$30*M245,0)</f>
+        <f>IF(A245=1,MIN(Variables!$B$32,260)*M245+Variables!$B$31*Variables!$B$2,IF(MOD(A245-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A245-1))*M245,0))-IF(A245=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD245" s="12">
@@ -32267,7 +32282,7 @@
         <v/>
       </c>
       <c r="AC246" s="11">
-        <f>IF(MOD(A246-1,Variables!$B$30)=0,Variables!$B$30*M246,0)</f>
+        <f>IF(A246=1,MIN(Variables!$B$32,260)*M246+Variables!$B$31*Variables!$B$2,IF(MOD(A246-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A246-1))*M246,0))-IF(A246=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD246" s="12">
@@ -32392,7 +32407,7 @@
         <v/>
       </c>
       <c r="AC247" s="11">
-        <f>IF(MOD(A247-1,Variables!$B$30)=0,Variables!$B$30*M247,0)</f>
+        <f>IF(A247=1,MIN(Variables!$B$32,260)*M247+Variables!$B$31*Variables!$B$2,IF(MOD(A247-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A247-1))*M247,0))-IF(A247=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD247" s="12">
@@ -32517,7 +32532,7 @@
         <v/>
       </c>
       <c r="AC248" s="11">
-        <f>IF(MOD(A248-1,Variables!$B$30)=0,Variables!$B$30*M248,0)</f>
+        <f>IF(A248=1,MIN(Variables!$B$32,260)*M248+Variables!$B$31*Variables!$B$2,IF(MOD(A248-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A248-1))*M248,0))-IF(A248=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD248" s="12">
@@ -32642,7 +32657,7 @@
         <v/>
       </c>
       <c r="AC249" s="11">
-        <f>IF(MOD(A249-1,Variables!$B$30)=0,Variables!$B$30*M249,0)</f>
+        <f>IF(A249=1,MIN(Variables!$B$32,260)*M249+Variables!$B$31*Variables!$B$2,IF(MOD(A249-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A249-1))*M249,0))-IF(A249=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD249" s="12">
@@ -32767,7 +32782,7 @@
         <v/>
       </c>
       <c r="AC250" s="11">
-        <f>IF(MOD(A250-1,Variables!$B$30)=0,Variables!$B$30*M250,0)</f>
+        <f>IF(A250=1,MIN(Variables!$B$32,260)*M250+Variables!$B$31*Variables!$B$2,IF(MOD(A250-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A250-1))*M250,0))-IF(A250=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD250" s="12">
@@ -32892,7 +32907,7 @@
         <v/>
       </c>
       <c r="AC251" s="11">
-        <f>IF(MOD(A251-1,Variables!$B$30)=0,Variables!$B$30*M251,0)</f>
+        <f>IF(A251=1,MIN(Variables!$B$32,260)*M251+Variables!$B$31*Variables!$B$2,IF(MOD(A251-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A251-1))*M251,0))-IF(A251=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD251" s="12">
@@ -33017,7 +33032,7 @@
         <v/>
       </c>
       <c r="AC252" s="11">
-        <f>IF(MOD(A252-1,Variables!$B$30)=0,Variables!$B$30*M252,0)</f>
+        <f>IF(A252=1,MIN(Variables!$B$32,260)*M252+Variables!$B$31*Variables!$B$2,IF(MOD(A252-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A252-1))*M252,0))-IF(A252=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD252" s="12">
@@ -33142,7 +33157,7 @@
         <v/>
       </c>
       <c r="AC253" s="11">
-        <f>IF(MOD(A253-1,Variables!$B$30)=0,Variables!$B$30*M253,0)</f>
+        <f>IF(A253=1,MIN(Variables!$B$32,260)*M253+Variables!$B$31*Variables!$B$2,IF(MOD(A253-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A253-1))*M253,0))-IF(A253=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD253" s="12">
@@ -33267,7 +33282,7 @@
         <v/>
       </c>
       <c r="AC254" s="11">
-        <f>IF(MOD(A254-1,Variables!$B$30)=0,Variables!$B$30*M254,0)</f>
+        <f>IF(A254=1,MIN(Variables!$B$32,260)*M254+Variables!$B$31*Variables!$B$2,IF(MOD(A254-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A254-1))*M254,0))-IF(A254=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD254" s="12">
@@ -33392,7 +33407,7 @@
         <v/>
       </c>
       <c r="AC255" s="11">
-        <f>IF(MOD(A255-1,Variables!$B$30)=0,Variables!$B$30*M255,0)</f>
+        <f>IF(A255=1,MIN(Variables!$B$32,260)*M255+Variables!$B$31*Variables!$B$2,IF(MOD(A255-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A255-1))*M255,0))-IF(A255=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD255" s="12">
@@ -33517,7 +33532,7 @@
         <v/>
       </c>
       <c r="AC256" s="11">
-        <f>IF(MOD(A256-1,Variables!$B$30)=0,Variables!$B$30*M256,0)</f>
+        <f>IF(A256=1,MIN(Variables!$B$32,260)*M256+Variables!$B$31*Variables!$B$2,IF(MOD(A256-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A256-1))*M256,0))-IF(A256=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD256" s="12">
@@ -33642,7 +33657,7 @@
         <v/>
       </c>
       <c r="AC257" s="11">
-        <f>IF(MOD(A257-1,Variables!$B$30)=0,Variables!$B$30*M257,0)</f>
+        <f>IF(A257=1,MIN(Variables!$B$32,260)*M257+Variables!$B$31*Variables!$B$2,IF(MOD(A257-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A257-1))*M257,0))-IF(A257=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD257" s="12">
@@ -33767,7 +33782,7 @@
         <v/>
       </c>
       <c r="AC258" s="11">
-        <f>IF(MOD(A258-1,Variables!$B$30)=0,Variables!$B$30*M258,0)</f>
+        <f>IF(A258=1,MIN(Variables!$B$32,260)*M258+Variables!$B$31*Variables!$B$2,IF(MOD(A258-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A258-1))*M258,0))-IF(A258=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD258" s="12">
@@ -33892,7 +33907,7 @@
         <v/>
       </c>
       <c r="AC259" s="11">
-        <f>IF(MOD(A259-1,Variables!$B$30)=0,Variables!$B$30*M259,0)</f>
+        <f>IF(A259=1,MIN(Variables!$B$32,260)*M259+Variables!$B$31*Variables!$B$2,IF(MOD(A259-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A259-1))*M259,0))-IF(A259=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD259" s="12">
@@ -34017,7 +34032,7 @@
         <v/>
       </c>
       <c r="AC260" s="11">
-        <f>IF(MOD(A260-1,Variables!$B$30)=0,Variables!$B$30*M260,0)</f>
+        <f>IF(A260=1,MIN(Variables!$B$32,260)*M260+Variables!$B$31*Variables!$B$2,IF(MOD(A260-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A260-1))*M260,0))-IF(A260=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD260" s="12">
@@ -34142,7 +34157,7 @@
         <v/>
       </c>
       <c r="AC261" s="11">
-        <f>IF(MOD(A261-1,Variables!$B$30)=0,Variables!$B$30*M261,0)</f>
+        <f>IF(A261=1,MIN(Variables!$B$32,260)*M261+Variables!$B$31*Variables!$B$2,IF(MOD(A261-1-Variables!$B$32,Variables!$B$30)=0,MIN(Variables!$B$30,260-(A261-1))*M261,0))-IF(A261=260,Variables!$B$31*Variables!$B$2,0)</f>
         <v/>
       </c>
       <c r="AD261" s="12">
@@ -34165,7 +34180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -34325,160 +34340,181 @@
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>6. CASH FLOW: fees are billed in N-week lumps, paid upfront (default 4), so cash</t>
+          <t>6. CASH FLOW: prepay weeks are paid up front on entry, then fees are billed in</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   dips every N weeks. Cash is spent first; once cash hits 0 the home value is drawn</t>
+          <t xml:space="preserve">   N-week lumps paid in advance, so cash dips at the start of each billing block.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   down (the house must be sold or equity released at that point).</t>
+          <t xml:space="preserve">   A deposit is also held (illiquid) and returned in the final week. Cash is spent</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr"/>
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   first; once cash hits 0 the home value is drawn down (the house must be sold or</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   equity released at that point).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>7. INCOME vs CAPITAL: the upper/lower limits apply to CAPITAL only.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Income (alimony + pension) is used for the weekly contribution, not the thresholds.</t>
+          <t xml:space="preserve">   Income (total, including the PEA) is used for the weekly contribution, not the thresholds.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>8. MEANS-TEST REVIEW: when total wealth falls to the review threshold (default 60,000)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">   the council carries out the financial assessment, ahead of taking over the subsidy</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">   at the upper capital limit (36,750).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>9. 12-WEEK DISREGARD: the funding boundary uses TOTAL wealth (cash + home), so the</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">   home is counted from day one for 'when does the council take over'. The disregard</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">   still appears in the 'Assessed capital' column and would only matter if council</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">   funding began within the first 12 weeks (not the case here).</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>10. BILLING: fees are billed in N-week lumps, paid upfront (see 'Care home billing</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    period'). The 'Capital (assessment)' columns track wealth smoothly, so funding</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    milestones are unaffected by the lump timing; the Cash/Home columns show the</t>
+          <t>10. BILLING: 'prepay weeks' are paid up front on entry, then fees are billed in</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    lumpy cash-flow (and the extra upfront buffer needed).</t>
+          <t xml:space="preserve">    N-week lumps paid in advance (see 'Care home billing period'); the deposit is</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr"/>
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    returned at the end. The 'Capital (assessment)' columns track wealth smoothly,</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    so funding milestones are unaffected by lump timing; the Cash/Home columns show</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    the lumpy cash-flow (and the extra upfront buffer needed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>Assumptions / caveats</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>- Rates and limits are as supplied; update them each April on the Variables sheet.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>- Income is counted in full and tax is ignored.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>- The home is assumed unoccupied (no qualifying relative) so it counts as capital.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>- A real local-authority financial assessment may vary; treat this as a planning model.</t>
         </is>

</xml_diff>